<commit_message>
Revise Meypak files so internal monitoring starts after the permit.
Periodic wastewater sampling is not required during the temporary operating certificate. The tracking workbook and report now start that schedule only after the environmental permit is issued.

Co-authored-by: iremalisan <iremalisan@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/cikti/Meypak_cevre_takip.xlsx
+++ b/cikti/Meypak_cevre_takip.xlsx
@@ -279,6 +279,12 @@
     <xf numFmtId="165" fontId="5" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -286,12 +292,6 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="165" fontId="5" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -360,11 +360,11 @@
     <xf numFmtId="0" fontId="7" fillId="16" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -1043,7 +1043,7 @@
       </c>
       <c r="B13" s="6" t="inlineStr">
         <is>
-          <t>Fiili debi 51-200 m³/gün bandında ise iki ayda bir. Tablo 5.9’daki üç parametrenin üçü de her seferinde bakılır.</t>
+          <t>Henüz yok. GFB aşamasında alınmaz. Atıksu deşarjı konulu çevre izin belgesi çıktıktan sonra, ekteki sıklıkla başlar. 51-200 m³/gün bandında beklenen sıklık iki ayda bir, parametreler KOİ, AKM ve pH.</t>
         </is>
       </c>
       <c r="C13" s="7" t="n"/>
@@ -1153,7 +1153,7 @@
     <row r="25" ht="36" customHeight="1">
       <c r="A25" s="14" t="inlineStr">
         <is>
-          <t>2  Eylül 2026 iç izleme alınmış deniyor; analiz raporu dosyada yok. Rapor bulunacak ya da numune hemen planlanacak. Kıyas: KOİ 150, AKM 200, pH 6-9.</t>
+          <t>2  İç izleme GFB aşamasında alınmaz. Tesisin iç izlemesi yoktur. Aylık rapordaki alındı cümlesi düzeltilecek. İlk numune, çevre izin belgesi çıktıktan sonra ekteki sıklıkla alınır.</t>
         </is>
       </c>
       <c r="B25" s="7" t="n"/>
@@ -1381,22 +1381,22 @@
       </c>
       <c r="C6" s="14" t="inlineStr">
         <is>
-          <t>Belge incelemesi</t>
+          <t>İşletme düzeltmesi</t>
         </is>
       </c>
       <c r="D6" s="14" t="inlineStr">
         <is>
-          <t>İç izleme alınmış deniyor, analiz raporu dosyada yok.</t>
+          <t>İç izleme eksikliği değildir. Tesisin periyodik iç izlemesi yoktur.</t>
         </is>
       </c>
       <c r="E6" s="14" t="inlineStr">
         <is>
-          <t>Rapor arşive girmemiş veya numune henüz oluşmamış.</t>
+          <t>GFB aşamasında iç izleme alınmaz. 24.09.2026 aylık rapordaki alındı cümlesi hatalıdır.</t>
         </is>
       </c>
       <c r="F6" s="14" t="inlineStr">
         <is>
-          <t>Raporu bul veya yeniden numune al. Y-02.</t>
+          <t>Sonraki aylık raporda cümle düzeltilecek. Numune, çevre izin belgesi çıktıktan sonra alınacak.</t>
         </is>
       </c>
       <c r="G6" s="14" t="inlineStr">
@@ -1405,11 +1405,11 @@
         </is>
       </c>
       <c r="H6" s="21" t="n">
-        <v>46302</v>
+        <v>46326</v>
       </c>
       <c r="I6" s="14" t="inlineStr">
         <is>
-          <t>Açık</t>
+          <t>Tamamlandı</t>
         </is>
       </c>
       <c r="J6" s="56" t="n"/>
@@ -1508,15 +1508,15 @@
           <t>U-05</t>
         </is>
       </c>
-      <c r="B9" s="50" t="n"/>
+      <c r="B9" s="49" t="n"/>
       <c r="C9" s="6" t="n"/>
       <c r="D9" s="6" t="n"/>
       <c r="E9" s="6" t="n"/>
       <c r="F9" s="6" t="n"/>
       <c r="G9" s="6" t="n"/>
-      <c r="H9" s="50" t="n"/>
+      <c r="H9" s="49" t="n"/>
       <c r="I9" s="6" t="n"/>
-      <c r="J9" s="50" t="n"/>
+      <c r="J9" s="49" t="n"/>
     </row>
     <row r="10" ht="22" customHeight="1">
       <c r="A10" s="6" t="inlineStr">
@@ -1524,15 +1524,15 @@
           <t>U-06</t>
         </is>
       </c>
-      <c r="B10" s="50" t="n"/>
+      <c r="B10" s="49" t="n"/>
       <c r="C10" s="6" t="n"/>
       <c r="D10" s="6" t="n"/>
       <c r="E10" s="6" t="n"/>
       <c r="F10" s="6" t="n"/>
       <c r="G10" s="6" t="n"/>
-      <c r="H10" s="50" t="n"/>
+      <c r="H10" s="49" t="n"/>
       <c r="I10" s="6" t="n"/>
-      <c r="J10" s="50" t="n"/>
+      <c r="J10" s="49" t="n"/>
     </row>
     <row r="11" ht="22" customHeight="1">
       <c r="A11" s="6" t="inlineStr">
@@ -1540,15 +1540,15 @@
           <t>U-07</t>
         </is>
       </c>
-      <c r="B11" s="50" t="n"/>
+      <c r="B11" s="49" t="n"/>
       <c r="C11" s="6" t="n"/>
       <c r="D11" s="6" t="n"/>
       <c r="E11" s="6" t="n"/>
       <c r="F11" s="6" t="n"/>
       <c r="G11" s="6" t="n"/>
-      <c r="H11" s="50" t="n"/>
+      <c r="H11" s="49" t="n"/>
       <c r="I11" s="6" t="n"/>
-      <c r="J11" s="50" t="n"/>
+      <c r="J11" s="49" t="n"/>
     </row>
     <row r="12" ht="22" customHeight="1">
       <c r="A12" s="6" t="inlineStr">
@@ -1556,15 +1556,15 @@
           <t>U-08</t>
         </is>
       </c>
-      <c r="B12" s="50" t="n"/>
+      <c r="B12" s="49" t="n"/>
       <c r="C12" s="6" t="n"/>
       <c r="D12" s="6" t="n"/>
       <c r="E12" s="6" t="n"/>
       <c r="F12" s="6" t="n"/>
       <c r="G12" s="6" t="n"/>
-      <c r="H12" s="50" t="n"/>
+      <c r="H12" s="49" t="n"/>
       <c r="I12" s="6" t="n"/>
-      <c r="J12" s="50" t="n"/>
+      <c r="J12" s="49" t="n"/>
     </row>
     <row r="13" ht="22" customHeight="1">
       <c r="A13" s="6" t="inlineStr">
@@ -1572,15 +1572,15 @@
           <t>U-09</t>
         </is>
       </c>
-      <c r="B13" s="50" t="n"/>
+      <c r="B13" s="49" t="n"/>
       <c r="C13" s="6" t="n"/>
       <c r="D13" s="6" t="n"/>
       <c r="E13" s="6" t="n"/>
       <c r="F13" s="6" t="n"/>
       <c r="G13" s="6" t="n"/>
-      <c r="H13" s="50" t="n"/>
+      <c r="H13" s="49" t="n"/>
       <c r="I13" s="6" t="n"/>
-      <c r="J13" s="50" t="n"/>
+      <c r="J13" s="49" t="n"/>
     </row>
     <row r="14" ht="22" customHeight="1">
       <c r="A14" s="6" t="inlineStr">
@@ -1588,15 +1588,15 @@
           <t>U-10</t>
         </is>
       </c>
-      <c r="B14" s="50" t="n"/>
+      <c r="B14" s="49" t="n"/>
       <c r="C14" s="6" t="n"/>
       <c r="D14" s="6" t="n"/>
       <c r="E14" s="6" t="n"/>
       <c r="F14" s="6" t="n"/>
       <c r="G14" s="6" t="n"/>
-      <c r="H14" s="50" t="n"/>
+      <c r="H14" s="49" t="n"/>
       <c r="I14" s="6" t="n"/>
-      <c r="J14" s="50" t="n"/>
+      <c r="J14" s="49" t="n"/>
     </row>
     <row r="15" ht="22" customHeight="1">
       <c r="A15" s="6" t="inlineStr">
@@ -1604,15 +1604,15 @@
           <t>U-11</t>
         </is>
       </c>
-      <c r="B15" s="50" t="n"/>
+      <c r="B15" s="49" t="n"/>
       <c r="C15" s="6" t="n"/>
       <c r="D15" s="6" t="n"/>
       <c r="E15" s="6" t="n"/>
       <c r="F15" s="6" t="n"/>
       <c r="G15" s="6" t="n"/>
-      <c r="H15" s="50" t="n"/>
+      <c r="H15" s="49" t="n"/>
       <c r="I15" s="6" t="n"/>
-      <c r="J15" s="50" t="n"/>
+      <c r="J15" s="49" t="n"/>
     </row>
     <row r="16" ht="22" customHeight="1">
       <c r="A16" s="6" t="inlineStr">
@@ -1620,15 +1620,15 @@
           <t>U-12</t>
         </is>
       </c>
-      <c r="B16" s="50" t="n"/>
+      <c r="B16" s="49" t="n"/>
       <c r="C16" s="6" t="n"/>
       <c r="D16" s="6" t="n"/>
       <c r="E16" s="6" t="n"/>
       <c r="F16" s="6" t="n"/>
       <c r="G16" s="6" t="n"/>
-      <c r="H16" s="50" t="n"/>
+      <c r="H16" s="49" t="n"/>
       <c r="I16" s="6" t="n"/>
-      <c r="J16" s="50" t="n"/>
+      <c r="J16" s="49" t="n"/>
     </row>
     <row r="17" ht="22" customHeight="1">
       <c r="A17" s="6" t="inlineStr">
@@ -1636,15 +1636,15 @@
           <t>U-13</t>
         </is>
       </c>
-      <c r="B17" s="50" t="n"/>
+      <c r="B17" s="49" t="n"/>
       <c r="C17" s="6" t="n"/>
       <c r="D17" s="6" t="n"/>
       <c r="E17" s="6" t="n"/>
       <c r="F17" s="6" t="n"/>
       <c r="G17" s="6" t="n"/>
-      <c r="H17" s="50" t="n"/>
+      <c r="H17" s="49" t="n"/>
       <c r="I17" s="6" t="n"/>
-      <c r="J17" s="50" t="n"/>
+      <c r="J17" s="49" t="n"/>
     </row>
     <row r="18" ht="22" customHeight="1">
       <c r="A18" s="6" t="inlineStr">
@@ -1652,15 +1652,15 @@
           <t>U-14</t>
         </is>
       </c>
-      <c r="B18" s="50" t="n"/>
+      <c r="B18" s="49" t="n"/>
       <c r="C18" s="6" t="n"/>
       <c r="D18" s="6" t="n"/>
       <c r="E18" s="6" t="n"/>
       <c r="F18" s="6" t="n"/>
       <c r="G18" s="6" t="n"/>
-      <c r="H18" s="50" t="n"/>
+      <c r="H18" s="49" t="n"/>
       <c r="I18" s="6" t="n"/>
-      <c r="J18" s="50" t="n"/>
+      <c r="J18" s="49" t="n"/>
     </row>
     <row r="19" ht="22" customHeight="1">
       <c r="A19" s="6" t="inlineStr">
@@ -1668,15 +1668,15 @@
           <t>U-15</t>
         </is>
       </c>
-      <c r="B19" s="50" t="n"/>
+      <c r="B19" s="49" t="n"/>
       <c r="C19" s="6" t="n"/>
       <c r="D19" s="6" t="n"/>
       <c r="E19" s="6" t="n"/>
       <c r="F19" s="6" t="n"/>
       <c r="G19" s="6" t="n"/>
-      <c r="H19" s="50" t="n"/>
+      <c r="H19" s="49" t="n"/>
       <c r="I19" s="6" t="n"/>
-      <c r="J19" s="50" t="n"/>
+      <c r="J19" s="49" t="n"/>
     </row>
     <row r="20" ht="22" customHeight="1">
       <c r="A20" s="6" t="inlineStr">
@@ -1684,15 +1684,15 @@
           <t>U-16</t>
         </is>
       </c>
-      <c r="B20" s="50" t="n"/>
+      <c r="B20" s="49" t="n"/>
       <c r="C20" s="6" t="n"/>
       <c r="D20" s="6" t="n"/>
       <c r="E20" s="6" t="n"/>
       <c r="F20" s="6" t="n"/>
       <c r="G20" s="6" t="n"/>
-      <c r="H20" s="50" t="n"/>
+      <c r="H20" s="49" t="n"/>
       <c r="I20" s="6" t="n"/>
-      <c r="J20" s="50" t="n"/>
+      <c r="J20" s="49" t="n"/>
     </row>
     <row r="21" ht="22" customHeight="1">
       <c r="A21" s="6" t="inlineStr">
@@ -1700,15 +1700,15 @@
           <t>U-17</t>
         </is>
       </c>
-      <c r="B21" s="50" t="n"/>
+      <c r="B21" s="49" t="n"/>
       <c r="C21" s="6" t="n"/>
       <c r="D21" s="6" t="n"/>
       <c r="E21" s="6" t="n"/>
       <c r="F21" s="6" t="n"/>
       <c r="G21" s="6" t="n"/>
-      <c r="H21" s="50" t="n"/>
+      <c r="H21" s="49" t="n"/>
       <c r="I21" s="6" t="n"/>
-      <c r="J21" s="50" t="n"/>
+      <c r="J21" s="49" t="n"/>
     </row>
     <row r="22" ht="22" customHeight="1">
       <c r="A22" s="6" t="inlineStr">
@@ -1716,15 +1716,15 @@
           <t>U-18</t>
         </is>
       </c>
-      <c r="B22" s="50" t="n"/>
+      <c r="B22" s="49" t="n"/>
       <c r="C22" s="6" t="n"/>
       <c r="D22" s="6" t="n"/>
       <c r="E22" s="6" t="n"/>
       <c r="F22" s="6" t="n"/>
       <c r="G22" s="6" t="n"/>
-      <c r="H22" s="50" t="n"/>
+      <c r="H22" s="49" t="n"/>
       <c r="I22" s="6" t="n"/>
-      <c r="J22" s="50" t="n"/>
+      <c r="J22" s="49" t="n"/>
     </row>
     <row r="23" ht="22" customHeight="1">
       <c r="A23" s="6" t="inlineStr">
@@ -1732,15 +1732,15 @@
           <t>U-19</t>
         </is>
       </c>
-      <c r="B23" s="50" t="n"/>
+      <c r="B23" s="49" t="n"/>
       <c r="C23" s="6" t="n"/>
       <c r="D23" s="6" t="n"/>
       <c r="E23" s="6" t="n"/>
       <c r="F23" s="6" t="n"/>
       <c r="G23" s="6" t="n"/>
-      <c r="H23" s="50" t="n"/>
+      <c r="H23" s="49" t="n"/>
       <c r="I23" s="6" t="n"/>
-      <c r="J23" s="50" t="n"/>
+      <c r="J23" s="49" t="n"/>
     </row>
     <row r="24" ht="22" customHeight="1">
       <c r="A24" s="6" t="inlineStr">
@@ -1748,15 +1748,15 @@
           <t>U-20</t>
         </is>
       </c>
-      <c r="B24" s="50" t="n"/>
+      <c r="B24" s="49" t="n"/>
       <c r="C24" s="6" t="n"/>
       <c r="D24" s="6" t="n"/>
       <c r="E24" s="6" t="n"/>
       <c r="F24" s="6" t="n"/>
       <c r="G24" s="6" t="n"/>
-      <c r="H24" s="50" t="n"/>
+      <c r="H24" s="49" t="n"/>
       <c r="I24" s="6" t="n"/>
-      <c r="J24" s="50" t="n"/>
+      <c r="J24" s="49" t="n"/>
     </row>
     <row r="25" ht="22" customHeight="1">
       <c r="A25" s="6" t="inlineStr">
@@ -1764,15 +1764,15 @@
           <t>U-21</t>
         </is>
       </c>
-      <c r="B25" s="50" t="n"/>
+      <c r="B25" s="49" t="n"/>
       <c r="C25" s="6" t="n"/>
       <c r="D25" s="6" t="n"/>
       <c r="E25" s="6" t="n"/>
       <c r="F25" s="6" t="n"/>
       <c r="G25" s="6" t="n"/>
-      <c r="H25" s="50" t="n"/>
+      <c r="H25" s="49" t="n"/>
       <c r="I25" s="6" t="n"/>
-      <c r="J25" s="50" t="n"/>
+      <c r="J25" s="49" t="n"/>
     </row>
     <row r="26" ht="22" customHeight="1">
       <c r="A26" s="6" t="inlineStr">
@@ -1780,15 +1780,15 @@
           <t>U-22</t>
         </is>
       </c>
-      <c r="B26" s="50" t="n"/>
+      <c r="B26" s="49" t="n"/>
       <c r="C26" s="6" t="n"/>
       <c r="D26" s="6" t="n"/>
       <c r="E26" s="6" t="n"/>
       <c r="F26" s="6" t="n"/>
       <c r="G26" s="6" t="n"/>
-      <c r="H26" s="50" t="n"/>
+      <c r="H26" s="49" t="n"/>
       <c r="I26" s="6" t="n"/>
-      <c r="J26" s="50" t="n"/>
+      <c r="J26" s="49" t="n"/>
     </row>
     <row r="27" ht="22" customHeight="1">
       <c r="A27" s="6" t="inlineStr">
@@ -1796,15 +1796,15 @@
           <t>U-23</t>
         </is>
       </c>
-      <c r="B27" s="50" t="n"/>
+      <c r="B27" s="49" t="n"/>
       <c r="C27" s="6" t="n"/>
       <c r="D27" s="6" t="n"/>
       <c r="E27" s="6" t="n"/>
       <c r="F27" s="6" t="n"/>
       <c r="G27" s="6" t="n"/>
-      <c r="H27" s="50" t="n"/>
+      <c r="H27" s="49" t="n"/>
       <c r="I27" s="6" t="n"/>
-      <c r="J27" s="50" t="n"/>
+      <c r="J27" s="49" t="n"/>
     </row>
     <row r="28" ht="22" customHeight="1">
       <c r="A28" s="6" t="inlineStr">
@@ -1812,15 +1812,15 @@
           <t>U-24</t>
         </is>
       </c>
-      <c r="B28" s="50" t="n"/>
+      <c r="B28" s="49" t="n"/>
       <c r="C28" s="6" t="n"/>
       <c r="D28" s="6" t="n"/>
       <c r="E28" s="6" t="n"/>
       <c r="F28" s="6" t="n"/>
       <c r="G28" s="6" t="n"/>
-      <c r="H28" s="50" t="n"/>
+      <c r="H28" s="49" t="n"/>
       <c r="I28" s="6" t="n"/>
-      <c r="J28" s="50" t="n"/>
+      <c r="J28" s="49" t="n"/>
     </row>
     <row r="29" ht="22" customHeight="1">
       <c r="A29" s="6" t="inlineStr">
@@ -1828,15 +1828,15 @@
           <t>U-25</t>
         </is>
       </c>
-      <c r="B29" s="50" t="n"/>
+      <c r="B29" s="49" t="n"/>
       <c r="C29" s="6" t="n"/>
       <c r="D29" s="6" t="n"/>
       <c r="E29" s="6" t="n"/>
       <c r="F29" s="6" t="n"/>
       <c r="G29" s="6" t="n"/>
-      <c r="H29" s="50" t="n"/>
+      <c r="H29" s="49" t="n"/>
       <c r="I29" s="6" t="n"/>
-      <c r="J29" s="50" t="n"/>
+      <c r="J29" s="49" t="n"/>
     </row>
     <row r="30" ht="22" customHeight="1">
       <c r="A30" s="6" t="inlineStr">
@@ -1844,15 +1844,15 @@
           <t>U-26</t>
         </is>
       </c>
-      <c r="B30" s="50" t="n"/>
+      <c r="B30" s="49" t="n"/>
       <c r="C30" s="6" t="n"/>
       <c r="D30" s="6" t="n"/>
       <c r="E30" s="6" t="n"/>
       <c r="F30" s="6" t="n"/>
       <c r="G30" s="6" t="n"/>
-      <c r="H30" s="50" t="n"/>
+      <c r="H30" s="49" t="n"/>
       <c r="I30" s="6" t="n"/>
-      <c r="J30" s="50" t="n"/>
+      <c r="J30" s="49" t="n"/>
     </row>
     <row r="31" ht="22" customHeight="1">
       <c r="A31" s="6" t="inlineStr">
@@ -1860,15 +1860,15 @@
           <t>U-27</t>
         </is>
       </c>
-      <c r="B31" s="50" t="n"/>
+      <c r="B31" s="49" t="n"/>
       <c r="C31" s="6" t="n"/>
       <c r="D31" s="6" t="n"/>
       <c r="E31" s="6" t="n"/>
       <c r="F31" s="6" t="n"/>
       <c r="G31" s="6" t="n"/>
-      <c r="H31" s="50" t="n"/>
+      <c r="H31" s="49" t="n"/>
       <c r="I31" s="6" t="n"/>
-      <c r="J31" s="50" t="n"/>
+      <c r="J31" s="49" t="n"/>
     </row>
     <row r="32" ht="22" customHeight="1">
       <c r="A32" s="6" t="inlineStr">
@@ -1876,15 +1876,15 @@
           <t>U-28</t>
         </is>
       </c>
-      <c r="B32" s="50" t="n"/>
+      <c r="B32" s="49" t="n"/>
       <c r="C32" s="6" t="n"/>
       <c r="D32" s="6" t="n"/>
       <c r="E32" s="6" t="n"/>
       <c r="F32" s="6" t="n"/>
       <c r="G32" s="6" t="n"/>
-      <c r="H32" s="50" t="n"/>
+      <c r="H32" s="49" t="n"/>
       <c r="I32" s="6" t="n"/>
-      <c r="J32" s="50" t="n"/>
+      <c r="J32" s="49" t="n"/>
     </row>
     <row r="33" ht="22" customHeight="1">
       <c r="A33" s="6" t="inlineStr">
@@ -1892,15 +1892,15 @@
           <t>U-29</t>
         </is>
       </c>
-      <c r="B33" s="50" t="n"/>
+      <c r="B33" s="49" t="n"/>
       <c r="C33" s="6" t="n"/>
       <c r="D33" s="6" t="n"/>
       <c r="E33" s="6" t="n"/>
       <c r="F33" s="6" t="n"/>
       <c r="G33" s="6" t="n"/>
-      <c r="H33" s="50" t="n"/>
+      <c r="H33" s="49" t="n"/>
       <c r="I33" s="6" t="n"/>
-      <c r="J33" s="50" t="n"/>
+      <c r="J33" s="49" t="n"/>
     </row>
     <row r="34" ht="22" customHeight="1">
       <c r="A34" s="6" t="inlineStr">
@@ -1908,15 +1908,15 @@
           <t>U-30</t>
         </is>
       </c>
-      <c r="B34" s="50" t="n"/>
+      <c r="B34" s="49" t="n"/>
       <c r="C34" s="6" t="n"/>
       <c r="D34" s="6" t="n"/>
       <c r="E34" s="6" t="n"/>
       <c r="F34" s="6" t="n"/>
       <c r="G34" s="6" t="n"/>
-      <c r="H34" s="50" t="n"/>
+      <c r="H34" s="49" t="n"/>
       <c r="I34" s="6" t="n"/>
-      <c r="J34" s="50" t="n"/>
+      <c r="J34" s="49" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A4:J40"/>
@@ -1982,7 +1982,7 @@
       </c>
       <c r="B4" s="6" t="inlineStr">
         <is>
-          <t>Uygunluk iddiası ancak analiz raporu ve debi ile kurulur. Eylül 2026 numunesi ‘alındı’ cümlesi sonuç değildir.</t>
+          <t>GFB aşamasında periyodik iç izleme alınmaz. Tesisin iç izlemesi yoktur. İlk iç izleme, atıksu deşarjı konulu çevre izin belgesi çıktıktan sonra, ekte yazılan aralıkla başlar.</t>
         </is>
       </c>
     </row>
@@ -2052,7 +2052,7 @@
       </c>
       <c r="B11" s="6" t="inlineStr">
         <is>
-          <t>Fiili debi 51-200 m³/gün ise iç izleme iki ayda bir, ilin denetime esas asgari sıklığı altı ayda birdir. Sürekli 50 ve altında dört aya inmek il müdürlüğünün yazısını gerektirir.</t>
+          <t>İzin çıktıktan sonra, fiili debi 51-200 m³/gün ise iç izleme iki ayda bir, ilin denetime esas asgari sıklığı altı ayda birdir. Sıklık izin ekinde yazar. Ek, bu notu ezer.</t>
         </is>
       </c>
     </row>
@@ -2912,17 +2912,17 @@
       </c>
       <c r="B32" s="19" t="inlineStr">
         <is>
-          <t>04.09.2026 iç tetkik: numune alınmamış. 24.09.2026 aylık rapor: rapor döneminde numune alınmış.</t>
+          <t>Tesisin iç izlemesi yoktur. GFB yürürlükteyken periyodik iç izleme alınmaz. 24.09.2026 aylık raporda alındığı yazılmış; bu cümle hatalıdır.</t>
         </is>
       </c>
       <c r="C32" s="19" t="inlineStr">
         <is>
-          <t>İki rapor</t>
+          <t>İşletme düzeltmesi</t>
         </is>
       </c>
       <c r="D32" s="19" t="inlineStr">
         <is>
-          <t>Analiz raporu bu sete dahil değil. Sonuç görülmeden uygunluk yazılmaz.</t>
+          <t>İç izleme, çevre izin belgesi çıktıktan sonra ekteki aralıkla başlar. İzne esas numune ile periyodik iç izleme aynı kayıt değildir.</t>
         </is>
       </c>
     </row>
@@ -3469,54 +3469,54 @@
       </c>
     </row>
     <row r="6" ht="78" customHeight="1">
-      <c r="A6" s="14" t="inlineStr">
+      <c r="A6" s="22" t="inlineStr">
         <is>
           <t>Y-02</t>
         </is>
       </c>
-      <c r="B6" s="14" t="inlineStr">
-        <is>
-          <t>Kritik</t>
-        </is>
-      </c>
-      <c r="C6" s="14" t="inlineStr">
+      <c r="B6" s="22" t="inlineStr">
+        <is>
+          <t>Düşük</t>
+        </is>
+      </c>
+      <c r="C6" s="22" t="inlineStr">
         <is>
           <t>İç izleme</t>
         </is>
       </c>
-      <c r="D6" s="14" t="inlineStr">
-        <is>
-          <t>Eylül 2026 analiz raporu</t>
-        </is>
-      </c>
-      <c r="E6" s="14" t="inlineStr">
-        <is>
-          <t>Aylık raporda numune alındığı, iç tetkikte alınmadığı yazıyor. Analiz raporunu, numune tutanağını ve o günkü debiyi bulun. KOİ 150 mg/L, AKM 200 mg/L ve pH 6-9 ile kıyaslayın. Aşım varsa il müdürlüğüne bildirim ve on iş günü içindeki iki ek numune dosyada mı bakın. Rapor yoksa yetkili laboratuvarla 2 saatlik kompozit numuneyi bu hafta planlayın.</t>
-        </is>
-      </c>
-      <c r="F6" s="14" t="inlineStr">
-        <is>
-          <t>04.09 iç tetkik 6.1.7 ve 24.09 aylık B.1.6</t>
-        </is>
-      </c>
-      <c r="G6" s="14" t="inlineStr">
+      <c r="D6" s="22" t="inlineStr">
+        <is>
+          <t>GFB aşamasında iç izleme yok</t>
+        </is>
+      </c>
+      <c r="E6" s="22" t="inlineStr">
+        <is>
+          <t>Tesisin periyodik iç izlemesi yoktur ve GFB yürürlükteyken alınmaz. İç izleme, atıksu deşarjı konulu çevre izin belgesi düzenlendikten sonra, belgenin ekindeki aralıkla başlar. 24.09.2026 aylık rapordaki iç izleme numunesi alınmıştır cümlesini sonraki raporda düzeltin. İzne esas numune ile periyodik iç izleme aynı şey değildir.</t>
+        </is>
+      </c>
+      <c r="F6" s="22" t="inlineStr">
+        <is>
+          <t>İşletme beyanı ve Numune Alma Tebliği madde 4/3</t>
+        </is>
+      </c>
+      <c r="G6" s="22" t="inlineStr">
         <is>
           <t>Çevre görevlisi</t>
         </is>
       </c>
-      <c r="H6" s="21" t="n">
-        <v>46302</v>
-      </c>
-      <c r="I6" s="14" t="inlineStr">
+      <c r="H6" s="23" t="n">
+        <v>46326</v>
+      </c>
+      <c r="I6" s="22" t="inlineStr">
         <is>
           <t>Açık</t>
         </is>
       </c>
-      <c r="J6" s="21" t="n"/>
-      <c r="K6" s="14" t="n"/>
-      <c r="L6" s="14" t="inlineStr">
-        <is>
-          <t>Sonuç görülmeden ‘limitlere uygun’ cümlesi rapora yazılmayacak.</t>
+      <c r="J6" s="23" t="n"/>
+      <c r="K6" s="22" t="n"/>
+      <c r="L6" s="22" t="inlineStr">
+        <is>
+          <t>İzin belgesi çıktığında ilk satıra belge tarihini yazın. 51-200 m³/gün için beklenen sıklık iki ayda birdir. Ek farklıysa ek uygulanır.</t>
         </is>
       </c>
     </row>
@@ -3625,312 +3625,312 @@
       </c>
     </row>
     <row r="9" ht="78" customHeight="1">
-      <c r="A9" s="22" t="inlineStr">
+      <c r="A9" s="24" t="inlineStr">
         <is>
           <t>Y-05</t>
         </is>
       </c>
-      <c r="B9" s="22" t="inlineStr">
+      <c r="B9" s="24" t="inlineStr">
         <is>
           <t>Yüksek</t>
         </is>
       </c>
-      <c r="C9" s="22" t="inlineStr">
+      <c r="C9" s="24" t="inlineStr">
         <is>
           <t>İzin</t>
         </is>
       </c>
-      <c r="D9" s="22" t="inlineStr">
+      <c r="D9" s="24" t="inlineStr">
         <is>
           <t>Çevre izin çıktısı ve eki</t>
         </is>
       </c>
-      <c r="E9" s="22" t="inlineStr">
+      <c r="E9" s="24" t="inlineStr">
         <is>
           <t>e-İzin’den atıksu deşarjı belge çıktısını ve ekini indirin. Ekteki debi, tablo, parametre, izleme sıklığı ve varsa ilave şart bu dosyadaki değerlerin önüne geçer. GFB 26.08.2027’de biter. Belge henüz oluşmamışsa GFB süresinde izin sürecini tamamlayın.</t>
         </is>
       </c>
-      <c r="F9" s="22" t="inlineStr">
+      <c r="F9" s="24" t="inlineStr">
         <is>
           <t>GFB 3069574032.1.1 ve uygunluk yazısı</t>
         </is>
       </c>
-      <c r="G9" s="22" t="inlineStr">
+      <c r="G9" s="24" t="inlineStr">
         <is>
           <t>Çevre görevlisi</t>
         </is>
       </c>
-      <c r="H9" s="23" t="n">
+      <c r="H9" s="25" t="n">
         <v>46310</v>
       </c>
-      <c r="I9" s="22" t="inlineStr">
+      <c r="I9" s="24" t="inlineStr">
         <is>
           <t>Açık</t>
         </is>
       </c>
-      <c r="J9" s="23" t="n"/>
-      <c r="K9" s="22" t="n"/>
-      <c r="L9" s="22" t="inlineStr">
+      <c r="J9" s="25" t="n"/>
+      <c r="K9" s="24" t="n"/>
+      <c r="L9" s="24" t="inlineStr">
         <is>
           <t>Uygunluk yazısı ile beş yıllık belge aynı evrak değildir.</t>
         </is>
       </c>
     </row>
     <row r="10" ht="78" customHeight="1">
-      <c r="A10" s="22" t="inlineStr">
+      <c r="A10" s="24" t="inlineStr">
         <is>
           <t>Y-06</t>
         </is>
       </c>
-      <c r="B10" s="22" t="inlineStr">
+      <c r="B10" s="24" t="inlineStr">
         <is>
           <t>Yüksek</t>
         </is>
       </c>
-      <c r="C10" s="22" t="inlineStr">
+      <c r="C10" s="24" t="inlineStr">
         <is>
           <t>Su temini</t>
         </is>
       </c>
-      <c r="D10" s="22" t="inlineStr">
+      <c r="D10" s="24" t="inlineStr">
         <is>
           <t>DSİ yeraltı suyu belgesi</t>
         </is>
       </c>
-      <c r="E10" s="22" t="inlineStr">
+      <c r="E10" s="24" t="inlineStr">
         <is>
           <t>Kuyu kullanılıyor ve belge dosyada yok. DSİ arama veya kullanma belgesini ya da tahsis yazısını isteyin. Yoksa başvuru başlatın. Kuyu sayacını okuyup SuDengesi sayfasına işleyin.</t>
         </is>
       </c>
-      <c r="F10" s="22" t="inlineStr">
+      <c r="F10" s="24" t="inlineStr">
         <is>
           <t>Aylık B.1.7, iç tetkik 6.1.7</t>
         </is>
       </c>
-      <c r="G10" s="22" t="inlineStr">
+      <c r="G10" s="24" t="inlineStr">
         <is>
           <t>İşletme</t>
         </is>
       </c>
-      <c r="H10" s="23" t="n">
+      <c r="H10" s="25" t="n">
         <v>46326</v>
       </c>
-      <c r="I10" s="22" t="inlineStr">
+      <c r="I10" s="24" t="inlineStr">
         <is>
           <t>Açık</t>
         </is>
       </c>
-      <c r="J10" s="23" t="n"/>
-      <c r="K10" s="22" t="n"/>
-      <c r="L10" s="22" t="inlineStr">
+      <c r="J10" s="25" t="n"/>
+      <c r="K10" s="24" t="n"/>
+      <c r="L10" s="24" t="inlineStr">
         <is>
           <t>Belge yokken kuyu debisini su dengesinden düşmeyin; ölçün ve ayrıca işaretleyin.</t>
         </is>
       </c>
     </row>
     <row r="11" ht="78" customHeight="1">
-      <c r="A11" s="22" t="inlineStr">
+      <c r="A11" s="24" t="inlineStr">
         <is>
           <t>Y-07</t>
         </is>
       </c>
-      <c r="B11" s="22" t="inlineStr">
+      <c r="B11" s="24" t="inlineStr">
         <is>
           <t>Yüksek</t>
         </is>
       </c>
-      <c r="C11" s="22" t="inlineStr">
+      <c r="C11" s="24" t="inlineStr">
         <is>
           <t>Debi</t>
         </is>
       </c>
-      <c r="D11" s="22" t="inlineStr">
+      <c r="D11" s="24" t="inlineStr">
         <is>
           <t>Günlük debi defteri</t>
         </is>
       </c>
-      <c r="E11" s="22" t="inlineStr">
+      <c r="E11" s="24" t="inlineStr">
         <is>
           <t>Giriş ve deşarj debisini GunlukIsletme sayfasına her gün yazın. 90 m³/gün aşımı kapasite ihlalidir. Fiili debi sürekli 50 m³/gün ve altında kalırsa izleme dört aya ancak il müdürlüğünün yazısıyla iner.</t>
         </is>
       </c>
-      <c r="F11" s="22" t="inlineStr">
+      <c r="F11" s="24" t="inlineStr">
         <is>
           <t>Kimlik kapasitesi 90 m³/gün</t>
         </is>
       </c>
-      <c r="G11" s="22" t="inlineStr">
+      <c r="G11" s="24" t="inlineStr">
         <is>
           <t>Tesis işletmecisi</t>
         </is>
       </c>
-      <c r="H11" s="23" t="n">
+      <c r="H11" s="25" t="n">
         <v>46310</v>
       </c>
-      <c r="I11" s="22" t="inlineStr">
+      <c r="I11" s="24" t="inlineStr">
         <is>
           <t>Açık</t>
         </is>
       </c>
-      <c r="J11" s="23" t="n"/>
-      <c r="K11" s="22" t="n"/>
-      <c r="L11" s="22" t="inlineStr">
+      <c r="J11" s="25" t="n"/>
+      <c r="K11" s="24" t="n"/>
+      <c r="L11" s="24" t="inlineStr">
         <is>
           <t>Su sayaçları (şebeke ve kuyu) ay sonunda SuDengesi’ne taşınsın.</t>
         </is>
       </c>
     </row>
     <row r="12" ht="78" customHeight="1">
-      <c r="A12" s="22" t="inlineStr">
+      <c r="A12" s="24" t="inlineStr">
         <is>
           <t>Y-08</t>
         </is>
       </c>
-      <c r="B12" s="22" t="inlineStr">
+      <c r="B12" s="24" t="inlineStr">
         <is>
           <t>Yüksek</t>
         </is>
       </c>
-      <c r="C12" s="22" t="inlineStr">
+      <c r="C12" s="24" t="inlineStr">
         <is>
           <t>Sigorta</t>
         </is>
       </c>
-      <c r="D12" s="22" t="inlineStr">
+      <c r="D12" s="24" t="inlineStr">
         <is>
           <t>Tehlikeli atık mali sorumluluk sigortası</t>
         </is>
       </c>
-      <c r="E12" s="22" t="inlineStr">
+      <c r="E12" s="24" t="inlineStr">
         <is>
           <t>Poliçe 23.02.2027’de bitiyor. Poliçe PDF’sini dosyalayın. Ocak 2027’de yenileme teklifini alın. Teminat, tesisin tehlikeli atık kodlarını kapsasın.</t>
         </is>
       </c>
-      <c r="F12" s="22" t="inlineStr">
+      <c r="F12" s="24" t="inlineStr">
         <is>
           <t>İç tetkik 6.3.6</t>
         </is>
       </c>
-      <c r="G12" s="22" t="inlineStr">
+      <c r="G12" s="24" t="inlineStr">
         <is>
           <t>İşletme</t>
         </is>
       </c>
-      <c r="H12" s="23" t="n">
+      <c r="H12" s="25" t="n">
         <v>46402</v>
       </c>
-      <c r="I12" s="22" t="inlineStr">
+      <c r="I12" s="24" t="inlineStr">
         <is>
           <t>Açık</t>
         </is>
       </c>
-      <c r="J12" s="23" t="n"/>
-      <c r="K12" s="22" t="n"/>
-      <c r="L12" s="22" t="inlineStr">
+      <c r="J12" s="25" t="n"/>
+      <c r="K12" s="24" t="n"/>
+      <c r="L12" s="24" t="inlineStr">
         <is>
           <t>Poliçe numarası mevcut raporlarda yok.</t>
         </is>
       </c>
     </row>
     <row r="13" ht="78" customHeight="1">
-      <c r="A13" s="22" t="inlineStr">
+      <c r="A13" s="24" t="inlineStr">
         <is>
           <t>Y-09</t>
         </is>
       </c>
-      <c r="B13" s="22" t="inlineStr">
+      <c r="B13" s="24" t="inlineStr">
         <is>
           <t>Yüksek</t>
         </is>
       </c>
-      <c r="C13" s="22" t="inlineStr">
+      <c r="C13" s="24" t="inlineStr">
         <is>
           <t>Kapasite</t>
         </is>
       </c>
-      <c r="D13" s="22" t="inlineStr">
+      <c r="D13" s="24" t="inlineStr">
         <is>
           <t>Kapasite raporu yenileme</t>
         </is>
       </c>
-      <c r="E13" s="22" t="inlineStr">
+      <c r="E13" s="24" t="inlineStr">
         <is>
           <t>TOBB kapasite raporu 03.03.2027’de bitiyor. Yenilenince günlük tonajı ÇED kapsam dışı kararı, Ek-1 madde 7.9 eşiği (100 ton/gün) ve KSTK eşiği ile yeniden karşılaştırın.</t>
         </is>
       </c>
-      <c r="F13" s="22" t="inlineStr">
+      <c r="F13" s="24" t="inlineStr">
         <is>
           <t>13.03.2025 / 150437</t>
         </is>
       </c>
-      <c r="G13" s="22" t="inlineStr">
+      <c r="G13" s="24" t="inlineStr">
         <is>
           <t>İşletme</t>
         </is>
       </c>
-      <c r="H13" s="23" t="n">
+      <c r="H13" s="25" t="n">
         <v>46402</v>
       </c>
-      <c r="I13" s="22" t="inlineStr">
+      <c r="I13" s="24" t="inlineStr">
         <is>
           <t>Açık</t>
         </is>
       </c>
-      <c r="J13" s="23" t="n"/>
-      <c r="K13" s="22" t="n"/>
-      <c r="L13" s="22" t="inlineStr">
+      <c r="J13" s="25" t="n"/>
+      <c r="K13" s="24" t="n"/>
+      <c r="L13" s="24" t="inlineStr">
         <is>
           <t>Mumlama 26.880 ton/yıl. Günlük eşik, çalışma günü sayısına göre değişir.</t>
         </is>
       </c>
     </row>
     <row r="14" ht="78" customHeight="1">
-      <c r="A14" s="22" t="inlineStr">
+      <c r="A14" s="24" t="inlineStr">
         <is>
           <t>Y-10</t>
         </is>
       </c>
-      <c r="B14" s="22" t="inlineStr">
+      <c r="B14" s="24" t="inlineStr">
         <is>
           <t>Yüksek</t>
         </is>
       </c>
-      <c r="C14" s="22" t="inlineStr">
+      <c r="C14" s="24" t="inlineStr">
         <is>
           <t>Personel sayısı</t>
         </is>
       </c>
-      <c r="D14" s="22" t="inlineStr">
+      <c r="D14" s="24" t="inlineStr">
         <is>
           <t>49 ile 60 çelişkisi</t>
         </is>
       </c>
-      <c r="E14" s="22" t="inlineStr">
+      <c r="E14" s="24" t="inlineStr">
         <is>
           <t>SGK hizmet listesinden güncel çalışan sayısını alın. İç tetkikteki su verimliliği muafiyeti 50 kişinin altına bağlanmış; aynı rapor toplamı 60. Sayı 50 ve üzerindeyse Su Verimliliği Yönetmeliği Ek-2 yükümlülüğünü yeniden değerlendirin.</t>
         </is>
       </c>
-      <c r="F14" s="22" t="inlineStr">
+      <c r="F14" s="24" t="inlineStr">
         <is>
           <t>Aylık rapor A bölümü ve iç tetkik 1 ve 6.13</t>
         </is>
       </c>
-      <c r="G14" s="22" t="inlineStr">
+      <c r="G14" s="24" t="inlineStr">
         <is>
           <t>Danışman</t>
         </is>
       </c>
-      <c r="H14" s="23" t="n">
+      <c r="H14" s="25" t="n">
         <v>46326</v>
       </c>
-      <c r="I14" s="22" t="inlineStr">
+      <c r="I14" s="24" t="inlineStr">
         <is>
           <t>Açık</t>
         </is>
       </c>
-      <c r="J14" s="23" t="n"/>
-      <c r="K14" s="22" t="n"/>
-      <c r="L14" s="22" t="inlineStr">
+      <c r="J14" s="25" t="n"/>
+      <c r="K14" s="24" t="n"/>
+      <c r="L14" s="24" t="inlineStr">
         <is>
           <t>Muafiyet cümlesi personel netleşmeden tekrar yazılmasın.</t>
         </is>
@@ -3972,7 +3972,7 @@
           <t>Tesis işletmecisi</t>
         </is>
       </c>
-      <c r="H15" s="24" t="n">
+      <c r="H15" s="26" t="n">
         <v>46310</v>
       </c>
       <c r="I15" s="19" t="inlineStr">
@@ -3980,7 +3980,7 @@
           <t>Açık</t>
         </is>
       </c>
-      <c r="J15" s="24" t="n"/>
+      <c r="J15" s="26" t="n"/>
       <c r="K15" s="19" t="n"/>
       <c r="L15" s="19" t="inlineStr">
         <is>
@@ -4024,7 +4024,7 @@
           <t>İşletme</t>
         </is>
       </c>
-      <c r="H16" s="24" t="n">
+      <c r="H16" s="26" t="n">
         <v>46326</v>
       </c>
       <c r="I16" s="19" t="inlineStr">
@@ -4032,7 +4032,7 @@
           <t>Açık</t>
         </is>
       </c>
-      <c r="J16" s="24" t="n"/>
+      <c r="J16" s="26" t="n"/>
       <c r="K16" s="19" t="n"/>
       <c r="L16" s="19" t="inlineStr">
         <is>
@@ -4076,7 +4076,7 @@
           <t>Çevre görevlisi</t>
         </is>
       </c>
-      <c r="H17" s="24" t="n">
+      <c r="H17" s="26" t="n">
         <v>46326</v>
       </c>
       <c r="I17" s="19" t="inlineStr">
@@ -4084,7 +4084,7 @@
           <t>Açık</t>
         </is>
       </c>
-      <c r="J17" s="24" t="n"/>
+      <c r="J17" s="26" t="n"/>
       <c r="K17" s="19" t="n"/>
       <c r="L17" s="19" t="inlineStr">
         <is>
@@ -4128,7 +4128,7 @@
           <t>Danışman</t>
         </is>
       </c>
-      <c r="H18" s="24" t="n">
+      <c r="H18" s="26" t="n">
         <v>46326</v>
       </c>
       <c r="I18" s="19" t="inlineStr">
@@ -4136,7 +4136,7 @@
           <t>Açık</t>
         </is>
       </c>
-      <c r="J18" s="24" t="n"/>
+      <c r="J18" s="26" t="n"/>
       <c r="K18" s="19" t="n"/>
       <c r="L18" s="19" t="inlineStr">
         <is>
@@ -4180,7 +4180,7 @@
           <t>Danışman</t>
         </is>
       </c>
-      <c r="H19" s="24" t="n">
+      <c r="H19" s="26" t="n">
         <v>46341</v>
       </c>
       <c r="I19" s="19" t="inlineStr">
@@ -4188,7 +4188,7 @@
           <t>Açık</t>
         </is>
       </c>
-      <c r="J19" s="24" t="n"/>
+      <c r="J19" s="26" t="n"/>
       <c r="K19" s="19" t="n"/>
       <c r="L19" s="19" t="inlineStr">
         <is>
@@ -4232,7 +4232,7 @@
           <t>Danışman</t>
         </is>
       </c>
-      <c r="H20" s="24" t="n">
+      <c r="H20" s="26" t="n">
         <v>46356</v>
       </c>
       <c r="I20" s="19" t="inlineStr">
@@ -4240,7 +4240,7 @@
           <t>Açık</t>
         </is>
       </c>
-      <c r="J20" s="24" t="n"/>
+      <c r="J20" s="26" t="n"/>
       <c r="K20" s="19" t="n"/>
       <c r="L20" s="19" t="inlineStr">
         <is>
@@ -4284,7 +4284,7 @@
           <t>İşletme</t>
         </is>
       </c>
-      <c r="H21" s="24" t="n">
+      <c r="H21" s="26" t="n">
         <v>46356</v>
       </c>
       <c r="I21" s="19" t="inlineStr">
@@ -4292,7 +4292,7 @@
           <t>Açık</t>
         </is>
       </c>
-      <c r="J21" s="24" t="n"/>
+      <c r="J21" s="26" t="n"/>
       <c r="K21" s="19" t="n"/>
       <c r="L21" s="19" t="inlineStr">
         <is>
@@ -4336,7 +4336,7 @@
           <t>Çevre görevlisi</t>
         </is>
       </c>
-      <c r="H22" s="24" t="n">
+      <c r="H22" s="26" t="n">
         <v>46461</v>
       </c>
       <c r="I22" s="19" t="inlineStr">
@@ -4344,7 +4344,7 @@
           <t>Açık</t>
         </is>
       </c>
-      <c r="J22" s="24" t="n"/>
+      <c r="J22" s="26" t="n"/>
       <c r="K22" s="19" t="n"/>
       <c r="L22" s="19" t="inlineStr">
         <is>
@@ -4388,7 +4388,7 @@
           <t>Danışman</t>
         </is>
       </c>
-      <c r="H23" s="24" t="n">
+      <c r="H23" s="26" t="n">
         <v>46341</v>
       </c>
       <c r="I23" s="19" t="inlineStr">
@@ -4396,7 +4396,7 @@
           <t>Açık</t>
         </is>
       </c>
-      <c r="J23" s="24" t="n"/>
+      <c r="J23" s="26" t="n"/>
       <c r="K23" s="19" t="n"/>
       <c r="L23" s="19" t="inlineStr"/>
     </row>
@@ -4436,7 +4436,7 @@
           <t>Tesis işletmecisi</t>
         </is>
       </c>
-      <c r="H24" s="24" t="n">
+      <c r="H24" s="26" t="n">
         <v>46310</v>
       </c>
       <c r="I24" s="19" t="inlineStr">
@@ -4444,7 +4444,7 @@
           <t>Açık</t>
         </is>
       </c>
-      <c r="J24" s="24" t="n"/>
+      <c r="J24" s="26" t="n"/>
       <c r="K24" s="19" t="n"/>
       <c r="L24" s="19" t="inlineStr">
         <is>
@@ -4453,100 +4453,100 @@
       </c>
     </row>
     <row r="25" ht="78" customHeight="1">
-      <c r="A25" s="25" t="inlineStr">
+      <c r="A25" s="22" t="inlineStr">
         <is>
           <t>Y-21</t>
         </is>
       </c>
-      <c r="B25" s="25" t="inlineStr">
+      <c r="B25" s="22" t="inlineStr">
         <is>
           <t>Düşük</t>
         </is>
       </c>
-      <c r="C25" s="25" t="inlineStr">
+      <c r="C25" s="22" t="inlineStr">
         <is>
           <t>Eğitim</t>
         </is>
       </c>
-      <c r="D25" s="25" t="inlineStr">
+      <c r="D25" s="22" t="inlineStr">
         <is>
           <t>24.09.2026 katılım formu</t>
         </is>
       </c>
-      <c r="E25" s="25" t="inlineStr">
+      <c r="E25" s="22" t="inlineStr">
         <is>
           <t>Aylık raporda çevre mevzuatı, genel atık ve sıfır atık eğitiminin 24.09.2026’da verildiği yazıyor. Yoklama ve konu başlığını dosyalayın. İç tetkik aynı eğitimi henüz verilecek diye yazmıştı.</t>
         </is>
       </c>
-      <c r="F25" s="25" t="inlineStr">
+      <c r="F25" s="22" t="inlineStr">
         <is>
           <t>Aylık rapor E.1</t>
         </is>
       </c>
-      <c r="G25" s="25" t="inlineStr">
+      <c r="G25" s="22" t="inlineStr">
         <is>
           <t>Çevre görevlisi</t>
         </is>
       </c>
-      <c r="H25" s="26" t="n">
+      <c r="H25" s="23" t="n">
         <v>46310</v>
       </c>
-      <c r="I25" s="25" t="inlineStr">
+      <c r="I25" s="22" t="inlineStr">
         <is>
           <t>Açık</t>
         </is>
       </c>
-      <c r="J25" s="26" t="n"/>
-      <c r="K25" s="25" t="n"/>
-      <c r="L25" s="25" t="inlineStr"/>
+      <c r="J25" s="23" t="n"/>
+      <c r="K25" s="22" t="n"/>
+      <c r="L25" s="22" t="inlineStr"/>
     </row>
     <row r="26" ht="78" customHeight="1">
-      <c r="A26" s="25" t="inlineStr">
+      <c r="A26" s="22" t="inlineStr">
         <is>
           <t>Y-22</t>
         </is>
       </c>
-      <c r="B26" s="25" t="inlineStr">
+      <c r="B26" s="22" t="inlineStr">
         <is>
           <t>Düşük</t>
         </is>
       </c>
-      <c r="C26" s="25" t="inlineStr">
+      <c r="C26" s="22" t="inlineStr">
         <is>
           <t>Sözleşme dosyası</t>
         </is>
       </c>
-      <c r="D26" s="25" t="inlineStr">
+      <c r="D26" s="22" t="inlineStr">
         <is>
           <t>Danışmanlık faturası ile sözleşme ayrılsın</t>
         </is>
       </c>
-      <c r="E26" s="25" t="inlineStr">
+      <c r="E26" s="22" t="inlineStr">
         <is>
           <t>Aylık raporda son fatura yerine 18.08.2026 sözleşme tarihi yazılmış. Sözleşme ve her ayın fatura numarası ayrı izlensin.</t>
         </is>
       </c>
-      <c r="F26" s="25" t="inlineStr">
+      <c r="F26" s="22" t="inlineStr">
         <is>
           <t>Aylık rapor A bölümü</t>
         </is>
       </c>
-      <c r="G26" s="25" t="inlineStr">
+      <c r="G26" s="22" t="inlineStr">
         <is>
           <t>KBRÇEV / işletme</t>
         </is>
       </c>
-      <c r="H26" s="26" t="n">
+      <c r="H26" s="23" t="n">
         <v>46326</v>
       </c>
-      <c r="I26" s="25" t="inlineStr">
+      <c r="I26" s="22" t="inlineStr">
         <is>
           <t>Açık</t>
         </is>
       </c>
-      <c r="J26" s="26" t="n"/>
-      <c r="K26" s="25" t="n"/>
-      <c r="L26" s="25" t="inlineStr"/>
+      <c r="J26" s="23" t="n"/>
+      <c r="K26" s="22" t="n"/>
+      <c r="L26" s="22" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A4:L26"/>
@@ -5454,12 +5454,12 @@
       </c>
       <c r="B23" s="18" t="inlineStr">
         <is>
-          <t>İç izleme analiz raporu (Eylül 2026)</t>
+          <t>Periyodik iç izleme</t>
         </is>
       </c>
       <c r="C23" s="18" t="inlineStr">
         <is>
-          <t>Alındı deniyor, rapor sette yok</t>
+          <t>Henüz başlamadı. GFB aşamasında alınmaz.</t>
         </is>
       </c>
       <c r="D23" s="28" t="n"/>
@@ -5472,19 +5472,19 @@
         <f>IF(E23="","Süresiz / olaya bağlı",IF(E23&lt;TODAY(),"SÜRESİ GEÇTİ",IF(E23-TODAY()&lt;=60,"60 GÜN İÇİNDE","GEÇERLİ")))</f>
         <v/>
       </c>
-      <c r="H23" s="34" t="inlineStr">
-        <is>
-          <t>Hayır</t>
+      <c r="H23" s="18" t="inlineStr">
+        <is>
+          <t>Henüz gerekmez</t>
         </is>
       </c>
       <c r="I23" s="18" t="inlineStr">
         <is>
-          <t>Hemen bulun veya yeniden alın</t>
+          <t>Çevre izin belgesi tarihinden sonra</t>
         </is>
       </c>
       <c r="J23" s="18" t="inlineStr">
         <is>
-          <t>Sonraki kampanya iki ay sonra.</t>
+          <t>İlk numune izin ekindeki sıklıkla alınır. 51-200 m³/gün bandında bu iki aydır.</t>
         </is>
       </c>
     </row>
@@ -5971,7 +5971,7 @@
           <t>Ünite</t>
         </is>
       </c>
-      <c r="B13" s="25" t="inlineStr">
+      <c r="B13" s="22" t="inlineStr">
         <is>
           <t>Izgara temiz, tutulan atık sahada birikmiyor</t>
         </is>
@@ -5996,7 +5996,7 @@
           <t>Ünite</t>
         </is>
       </c>
-      <c r="B14" s="25" t="inlineStr">
+      <c r="B14" s="22" t="inlineStr">
         <is>
           <t>Kum tutucu çalışıyor</t>
         </is>
@@ -6021,7 +6021,7 @@
           <t>Ünite</t>
         </is>
       </c>
-      <c r="B15" s="25" t="inlineStr">
+      <c r="B15" s="22" t="inlineStr">
         <is>
           <t>Dengeleme havuzu seviye ve karıştırması normal, taşma yok</t>
         </is>
@@ -6046,7 +6046,7 @@
           <t>Ünite</t>
         </is>
       </c>
-      <c r="B16" s="25" t="inlineStr">
+      <c r="B16" s="22" t="inlineStr">
         <is>
           <t>Havalandırmada çözünmüş oksijen, renk ve koku normal</t>
         </is>
@@ -6071,7 +6071,7 @@
           <t>Ünite</t>
         </is>
       </c>
-      <c r="B17" s="25" t="inlineStr">
+      <c r="B17" s="22" t="inlineStr">
         <is>
           <t>Çöktürme savağı temiz, çamur kaçışı yok</t>
         </is>
@@ -6096,7 +6096,7 @@
           <t>Ünite</t>
         </is>
       </c>
-      <c r="B18" s="25" t="inlineStr">
+      <c r="B18" s="22" t="inlineStr">
         <is>
           <t>Klor temas tankı devrede, doz kaydı var</t>
         </is>
@@ -6121,7 +6121,7 @@
           <t>Ünite</t>
         </is>
       </c>
-      <c r="B19" s="25" t="inlineStr">
+      <c r="B19" s="22" t="inlineStr">
         <is>
           <t>Yedek pompa veya blower arızası işletmeyi durdurmuyor</t>
         </is>
@@ -6273,7 +6273,7 @@
       </c>
       <c r="B25" s="19" t="inlineStr">
         <is>
-          <t>İç izleme kampanyası takvimde ve sonuç dosyada</t>
+          <t>GFB sürüyorsa iç izleme alınmamıştır. İzin çıktıysa kampanya zamanındadır</t>
         </is>
       </c>
       <c r="C25" s="37" t="n"/>
@@ -6298,7 +6298,7 @@
       </c>
       <c r="B26" s="19" t="inlineStr">
         <is>
-          <t>Son analiz KOİ, AKM ve pH limite uygun</t>
+          <t>İzin çıktıktan sonra son analiz KOİ, AKM ve pH limite uygundur</t>
         </is>
       </c>
       <c r="C26" s="37" t="n"/>
@@ -6323,7 +6323,7 @@
       </c>
       <c r="B27" s="19" t="inlineStr">
         <is>
-          <t>Aşım varsa bildirim ve on iş günü ek numuneleri dosyada</t>
+          <t>İç izleme aşımında bildirim ve on iş günü ek numuneleri dosyadadır</t>
         </is>
       </c>
       <c r="C27" s="37" t="n"/>
@@ -6471,7 +6471,7 @@
           <t>Kimyasal</t>
         </is>
       </c>
-      <c r="B33" s="22" t="inlineStr">
+      <c r="B33" s="24" t="inlineStr">
         <is>
           <t>Hipoklorit, mum ve diğer SDS’ler klasörde</t>
         </is>
@@ -6496,7 +6496,7 @@
           <t>Kimyasal</t>
         </is>
       </c>
-      <c r="B34" s="22" t="inlineStr">
+      <c r="B34" s="24" t="inlineStr">
         <is>
           <t>Dökülme kiti yerinde, zemin sızıntısı yok</t>
         </is>
@@ -6779,7 +6779,7 @@
     <row r="2" ht="32" customHeight="1">
       <c r="A2" s="15" t="inlineStr">
         <is>
-          <t>Yasal kıyas 2 saatlik kompozittir. Limitler: KOİ 150 mg/L, AKM 200 mg/L, pH 6-9. pH’de yüzde 20 payı yoktur. KOİ ve AKM anlık numunede limitin yüzde 20 fazlası yaptırıma esas değerlendirilir; iç izlemeyi anlık numuneyle kapatmayın. Aşımda il müdürlüğüne bildirim ve on iş günü içinde iki ek numune. Üç sonucun ortalaması yazılır.</t>
+          <t>GFB aşamasında bu sayfa boş kalır. Periyodik iç izleme, çevre izin belgesi çıktıktan sonra başlar. Yasal kıyas 2 saatlik kompozittir. Limitler: KOİ 150 mg/L, AKM 200 mg/L, pH 6-9. Aşımda il müdürlüğüne bildirim ve on iş günü içinde iki ek numune. Üç sonucun ortalaması yazılır.</t>
         </is>
       </c>
     </row>
@@ -6901,64 +6901,64 @@
       </c>
     </row>
     <row r="5" ht="32" customHeight="1">
-      <c r="A5" s="19" t="n">
+      <c r="A5" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="B5" s="19" t="inlineStr">
-        <is>
-          <t>Eylül 2026</t>
-        </is>
-      </c>
-      <c r="C5" s="24" t="n"/>
-      <c r="D5" s="19" t="inlineStr">
+      <c r="B5" s="6" t="inlineStr">
+        <is>
+          <t>İzin sonrası 1</t>
+        </is>
+      </c>
+      <c r="C5" s="49" t="n"/>
+      <c r="D5" s="6" t="inlineStr">
         <is>
           <t>2 saatlik kompozit</t>
         </is>
       </c>
-      <c r="E5" s="19" t="n"/>
-      <c r="F5" s="19" t="n"/>
-      <c r="G5" s="19" t="n"/>
-      <c r="H5" s="19" t="n"/>
-      <c r="I5" s="49" t="n">
+      <c r="E5" s="6" t="n"/>
+      <c r="F5" s="6" t="n"/>
+      <c r="G5" s="6" t="n"/>
+      <c r="H5" s="6" t="n"/>
+      <c r="I5" s="50" t="n">
         <v>150</v>
       </c>
-      <c r="J5" s="19">
+      <c r="J5" s="6">
         <f>IF(H5="","",IF(H5&lt;=I5,"UYGUN","AŞIM"))</f>
         <v/>
       </c>
-      <c r="K5" s="19" t="n"/>
-      <c r="L5" s="49" t="n">
+      <c r="K5" s="6" t="n"/>
+      <c r="L5" s="50" t="n">
         <v>200</v>
       </c>
-      <c r="M5" s="19">
+      <c r="M5" s="6">
         <f>IF(K5="","",IF(K5&lt;=L5,"UYGUN","AŞIM"))</f>
         <v/>
       </c>
-      <c r="N5" s="19" t="n"/>
-      <c r="O5" s="49" t="n">
+      <c r="N5" s="6" t="n"/>
+      <c r="O5" s="50" t="n">
         <v>6</v>
       </c>
-      <c r="P5" s="49" t="n">
+      <c r="P5" s="50" t="n">
         <v>9</v>
       </c>
-      <c r="Q5" s="19">
+      <c r="Q5" s="6">
         <f>IF(N5="","",IF(AND(N5&gt;=O5,N5&lt;=P5),"UYGUN","AŞIM"))</f>
         <v/>
       </c>
-      <c r="R5" s="19">
+      <c r="R5" s="6">
         <f>IF(COUNT(H5,K5,N5)&lt;3,"EKSİK",IF(OR(J5="AŞIM",M5="AŞIM",Q5="AŞIM"),"AŞIM","UYGUN"))</f>
         <v/>
       </c>
-      <c r="S5" s="19">
+      <c r="S5" s="6">
         <f>IF(R5="AŞIM","Evet",IF(R5="UYGUN","Hayır",""))</f>
         <v/>
       </c>
-      <c r="T5" s="24" t="n"/>
-      <c r="U5" s="19" t="n"/>
-      <c r="V5" s="19" t="n"/>
-      <c r="W5" s="19" t="inlineStr">
-        <is>
-          <t>Alındığı beyan edildi, rapor dosyada yok. Sonucu bu satıra işleyin.</t>
+      <c r="T5" s="49" t="n"/>
+      <c r="U5" s="6" t="n"/>
+      <c r="V5" s="6" t="n"/>
+      <c r="W5" s="6" t="inlineStr">
+        <is>
+          <t>GFB sürerken boş bırakın. Çevre izin belgesinin tarihini yazınca ilk numuneyi ekteki sıklığa göre planlayın.</t>
         </is>
       </c>
     </row>
@@ -6968,10 +6968,10 @@
       </c>
       <c r="B6" s="6" t="inlineStr">
         <is>
-          <t>Kasım 2026</t>
-        </is>
-      </c>
-      <c r="C6" s="50" t="n"/>
+          <t>2. kampanya</t>
+        </is>
+      </c>
+      <c r="C6" s="49" t="n"/>
       <c r="D6" s="6" t="inlineStr">
         <is>
           <t>2 saatlik kompozit</t>
@@ -6981,7 +6981,7 @@
       <c r="F6" s="6" t="n"/>
       <c r="G6" s="6" t="n"/>
       <c r="H6" s="6" t="n"/>
-      <c r="I6" s="49" t="n">
+      <c r="I6" s="50" t="n">
         <v>150</v>
       </c>
       <c r="J6" s="6">
@@ -6989,7 +6989,7 @@
         <v/>
       </c>
       <c r="K6" s="6" t="n"/>
-      <c r="L6" s="49" t="n">
+      <c r="L6" s="50" t="n">
         <v>200</v>
       </c>
       <c r="M6" s="6">
@@ -6997,10 +6997,10 @@
         <v/>
       </c>
       <c r="N6" s="6" t="n"/>
-      <c r="O6" s="49" t="n">
+      <c r="O6" s="50" t="n">
         <v>6</v>
       </c>
-      <c r="P6" s="49" t="n">
+      <c r="P6" s="50" t="n">
         <v>9</v>
       </c>
       <c r="Q6" s="6">
@@ -7015,12 +7015,12 @@
         <f>IF(R6="AŞIM","Evet",IF(R6="UYGUN","Hayır",""))</f>
         <v/>
       </c>
-      <c r="T6" s="50" t="n"/>
+      <c r="T6" s="49" t="n"/>
       <c r="U6" s="6" t="n"/>
       <c r="V6" s="6" t="n"/>
       <c r="W6" s="6" t="inlineStr">
         <is>
-          <t>Eylül numunesinden iki ay sonra. Tarih netleşince yazın.</t>
+          <t>İlk numuneden iki ay sonra. Ek başka süre verirse onu yazın.</t>
         </is>
       </c>
     </row>
@@ -7030,10 +7030,10 @@
       </c>
       <c r="B7" s="6" t="inlineStr">
         <is>
-          <t>Ocak 2027</t>
-        </is>
-      </c>
-      <c r="C7" s="50" t="n"/>
+          <t>3. kampanya</t>
+        </is>
+      </c>
+      <c r="C7" s="49" t="n"/>
       <c r="D7" s="6" t="inlineStr">
         <is>
           <t>2 saatlik kompozit</t>
@@ -7043,7 +7043,7 @@
       <c r="F7" s="6" t="n"/>
       <c r="G7" s="6" t="n"/>
       <c r="H7" s="6" t="n"/>
-      <c r="I7" s="49" t="n">
+      <c r="I7" s="50" t="n">
         <v>150</v>
       </c>
       <c r="J7" s="6">
@@ -7051,7 +7051,7 @@
         <v/>
       </c>
       <c r="K7" s="6" t="n"/>
-      <c r="L7" s="49" t="n">
+      <c r="L7" s="50" t="n">
         <v>200</v>
       </c>
       <c r="M7" s="6">
@@ -7059,10 +7059,10 @@
         <v/>
       </c>
       <c r="N7" s="6" t="n"/>
-      <c r="O7" s="49" t="n">
+      <c r="O7" s="50" t="n">
         <v>6</v>
       </c>
-      <c r="P7" s="49" t="n">
+      <c r="P7" s="50" t="n">
         <v>9</v>
       </c>
       <c r="Q7" s="6">
@@ -7077,7 +7077,7 @@
         <f>IF(R7="AŞIM","Evet",IF(R7="UYGUN","Hayır",""))</f>
         <v/>
       </c>
-      <c r="T7" s="50" t="n"/>
+      <c r="T7" s="49" t="n"/>
       <c r="U7" s="6" t="n"/>
       <c r="V7" s="6" t="n"/>
       <c r="W7" s="6" t="inlineStr"/>
@@ -7088,10 +7088,10 @@
       </c>
       <c r="B8" s="6" t="inlineStr">
         <is>
-          <t>Mart 2027</t>
-        </is>
-      </c>
-      <c r="C8" s="50" t="n"/>
+          <t>4. kampanya</t>
+        </is>
+      </c>
+      <c r="C8" s="49" t="n"/>
       <c r="D8" s="6" t="inlineStr">
         <is>
           <t>2 saatlik kompozit</t>
@@ -7101,7 +7101,7 @@
       <c r="F8" s="6" t="n"/>
       <c r="G8" s="6" t="n"/>
       <c r="H8" s="6" t="n"/>
-      <c r="I8" s="49" t="n">
+      <c r="I8" s="50" t="n">
         <v>150</v>
       </c>
       <c r="J8" s="6">
@@ -7109,7 +7109,7 @@
         <v/>
       </c>
       <c r="K8" s="6" t="n"/>
-      <c r="L8" s="49" t="n">
+      <c r="L8" s="50" t="n">
         <v>200</v>
       </c>
       <c r="M8" s="6">
@@ -7117,10 +7117,10 @@
         <v/>
       </c>
       <c r="N8" s="6" t="n"/>
-      <c r="O8" s="49" t="n">
+      <c r="O8" s="50" t="n">
         <v>6</v>
       </c>
-      <c r="P8" s="49" t="n">
+      <c r="P8" s="50" t="n">
         <v>9</v>
       </c>
       <c r="Q8" s="6">
@@ -7135,7 +7135,7 @@
         <f>IF(R8="AŞIM","Evet",IF(R8="UYGUN","Hayır",""))</f>
         <v/>
       </c>
-      <c r="T8" s="50" t="n"/>
+      <c r="T8" s="49" t="n"/>
       <c r="U8" s="6" t="n"/>
       <c r="V8" s="6" t="n"/>
       <c r="W8" s="6" t="inlineStr"/>
@@ -7146,10 +7146,10 @@
       </c>
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>Mayıs 2027</t>
-        </is>
-      </c>
-      <c r="C9" s="50" t="n"/>
+          <t>5. kampanya</t>
+        </is>
+      </c>
+      <c r="C9" s="49" t="n"/>
       <c r="D9" s="6" t="inlineStr">
         <is>
           <t>2 saatlik kompozit</t>
@@ -7159,7 +7159,7 @@
       <c r="F9" s="6" t="n"/>
       <c r="G9" s="6" t="n"/>
       <c r="H9" s="6" t="n"/>
-      <c r="I9" s="49" t="n">
+      <c r="I9" s="50" t="n">
         <v>150</v>
       </c>
       <c r="J9" s="6">
@@ -7167,7 +7167,7 @@
         <v/>
       </c>
       <c r="K9" s="6" t="n"/>
-      <c r="L9" s="49" t="n">
+      <c r="L9" s="50" t="n">
         <v>200</v>
       </c>
       <c r="M9" s="6">
@@ -7175,10 +7175,10 @@
         <v/>
       </c>
       <c r="N9" s="6" t="n"/>
-      <c r="O9" s="49" t="n">
+      <c r="O9" s="50" t="n">
         <v>6</v>
       </c>
-      <c r="P9" s="49" t="n">
+      <c r="P9" s="50" t="n">
         <v>9</v>
       </c>
       <c r="Q9" s="6">
@@ -7193,7 +7193,7 @@
         <f>IF(R9="AŞIM","Evet",IF(R9="UYGUN","Hayır",""))</f>
         <v/>
       </c>
-      <c r="T9" s="50" t="n"/>
+      <c r="T9" s="49" t="n"/>
       <c r="U9" s="6" t="n"/>
       <c r="V9" s="6" t="n"/>
       <c r="W9" s="6" t="inlineStr"/>
@@ -7204,10 +7204,10 @@
       </c>
       <c r="B10" s="6" t="inlineStr">
         <is>
-          <t>Temmuz 2027</t>
-        </is>
-      </c>
-      <c r="C10" s="50" t="n"/>
+          <t>6. kampanya</t>
+        </is>
+      </c>
+      <c r="C10" s="49" t="n"/>
       <c r="D10" s="6" t="inlineStr">
         <is>
           <t>2 saatlik kompozit</t>
@@ -7217,7 +7217,7 @@
       <c r="F10" s="6" t="n"/>
       <c r="G10" s="6" t="n"/>
       <c r="H10" s="6" t="n"/>
-      <c r="I10" s="49" t="n">
+      <c r="I10" s="50" t="n">
         <v>150</v>
       </c>
       <c r="J10" s="6">
@@ -7225,7 +7225,7 @@
         <v/>
       </c>
       <c r="K10" s="6" t="n"/>
-      <c r="L10" s="49" t="n">
+      <c r="L10" s="50" t="n">
         <v>200</v>
       </c>
       <c r="M10" s="6">
@@ -7233,10 +7233,10 @@
         <v/>
       </c>
       <c r="N10" s="6" t="n"/>
-      <c r="O10" s="49" t="n">
+      <c r="O10" s="50" t="n">
         <v>6</v>
       </c>
-      <c r="P10" s="49" t="n">
+      <c r="P10" s="50" t="n">
         <v>9</v>
       </c>
       <c r="Q10" s="6">
@@ -7251,7 +7251,7 @@
         <f>IF(R10="AŞIM","Evet",IF(R10="UYGUN","Hayır",""))</f>
         <v/>
       </c>
-      <c r="T10" s="50" t="n"/>
+      <c r="T10" s="49" t="n"/>
       <c r="U10" s="6" t="n"/>
       <c r="V10" s="6" t="n"/>
       <c r="W10" s="6" t="inlineStr"/>
@@ -7262,10 +7262,10 @@
       </c>
       <c r="B11" s="6" t="inlineStr">
         <is>
-          <t>Eylül 2027</t>
-        </is>
-      </c>
-      <c r="C11" s="50" t="n"/>
+          <t>7. kampanya</t>
+        </is>
+      </c>
+      <c r="C11" s="49" t="n"/>
       <c r="D11" s="6" t="inlineStr">
         <is>
           <t>2 saatlik kompozit</t>
@@ -7275,7 +7275,7 @@
       <c r="F11" s="6" t="n"/>
       <c r="G11" s="6" t="n"/>
       <c r="H11" s="6" t="n"/>
-      <c r="I11" s="49" t="n">
+      <c r="I11" s="50" t="n">
         <v>150</v>
       </c>
       <c r="J11" s="6">
@@ -7283,7 +7283,7 @@
         <v/>
       </c>
       <c r="K11" s="6" t="n"/>
-      <c r="L11" s="49" t="n">
+      <c r="L11" s="50" t="n">
         <v>200</v>
       </c>
       <c r="M11" s="6">
@@ -7291,10 +7291,10 @@
         <v/>
       </c>
       <c r="N11" s="6" t="n"/>
-      <c r="O11" s="49" t="n">
+      <c r="O11" s="50" t="n">
         <v>6</v>
       </c>
-      <c r="P11" s="49" t="n">
+      <c r="P11" s="50" t="n">
         <v>9</v>
       </c>
       <c r="Q11" s="6">
@@ -7309,12 +7309,12 @@
         <f>IF(R11="AŞIM","Evet",IF(R11="UYGUN","Hayır",""))</f>
         <v/>
       </c>
-      <c r="T11" s="50" t="n"/>
+      <c r="T11" s="49" t="n"/>
       <c r="U11" s="6" t="n"/>
       <c r="V11" s="6" t="n"/>
       <c r="W11" s="6" t="inlineStr">
         <is>
-          <t>GFB 26.08.2027’de biter. İzin eki farklı sıklık verirse takvimi eke göre değiştirin.</t>
+          <t>GFB 26.08.2027’ye kadar iç izleme alınmaz.</t>
         </is>
       </c>
     </row>
@@ -7329,7 +7329,7 @@
           <t>Ek numune</t>
         </is>
       </c>
-      <c r="C12" s="50" t="n"/>
+      <c r="C12" s="49" t="n"/>
       <c r="D12" s="6" t="inlineStr">
         <is>
           <t>2 saatlik kompozit</t>
@@ -7339,7 +7339,7 @@
       <c r="F12" s="6" t="n"/>
       <c r="G12" s="6" t="n"/>
       <c r="H12" s="6" t="n"/>
-      <c r="I12" s="25" t="n">
+      <c r="I12" s="22" t="n">
         <v>150</v>
       </c>
       <c r="J12" s="6">
@@ -7347,7 +7347,7 @@
         <v/>
       </c>
       <c r="K12" s="6" t="n"/>
-      <c r="L12" s="25" t="n">
+      <c r="L12" s="22" t="n">
         <v>200</v>
       </c>
       <c r="M12" s="6">
@@ -7355,10 +7355,10 @@
         <v/>
       </c>
       <c r="N12" s="6" t="n"/>
-      <c r="O12" s="25" t="n">
+      <c r="O12" s="22" t="n">
         <v>6</v>
       </c>
-      <c r="P12" s="25" t="n">
+      <c r="P12" s="22" t="n">
         <v>9</v>
       </c>
       <c r="Q12" s="6">
@@ -7373,7 +7373,7 @@
         <f>IF(R12="AŞIM","Evet",IF(R12="UYGUN","Hayır",""))</f>
         <v/>
       </c>
-      <c r="T12" s="50" t="n"/>
+      <c r="T12" s="49" t="n"/>
       <c r="U12" s="6" t="n"/>
       <c r="V12" s="6" t="n"/>
       <c r="W12" s="6" t="inlineStr">
@@ -7393,7 +7393,7 @@
           <t>Ek numune</t>
         </is>
       </c>
-      <c r="C13" s="50" t="n"/>
+      <c r="C13" s="49" t="n"/>
       <c r="D13" s="6" t="inlineStr">
         <is>
           <t>2 saatlik kompozit</t>
@@ -7403,7 +7403,7 @@
       <c r="F13" s="6" t="n"/>
       <c r="G13" s="6" t="n"/>
       <c r="H13" s="6" t="n"/>
-      <c r="I13" s="25" t="n">
+      <c r="I13" s="22" t="n">
         <v>150</v>
       </c>
       <c r="J13" s="6">
@@ -7411,7 +7411,7 @@
         <v/>
       </c>
       <c r="K13" s="6" t="n"/>
-      <c r="L13" s="25" t="n">
+      <c r="L13" s="22" t="n">
         <v>200</v>
       </c>
       <c r="M13" s="6">
@@ -7419,10 +7419,10 @@
         <v/>
       </c>
       <c r="N13" s="6" t="n"/>
-      <c r="O13" s="25" t="n">
+      <c r="O13" s="22" t="n">
         <v>6</v>
       </c>
-      <c r="P13" s="25" t="n">
+      <c r="P13" s="22" t="n">
         <v>9</v>
       </c>
       <c r="Q13" s="6">
@@ -7437,7 +7437,7 @@
         <f>IF(R13="AŞIM","Evet",IF(R13="UYGUN","Hayır",""))</f>
         <v/>
       </c>
-      <c r="T13" s="50" t="n"/>
+      <c r="T13" s="49" t="n"/>
       <c r="U13" s="6" t="n"/>
       <c r="V13" s="6" t="n"/>
       <c r="W13" s="6" t="inlineStr">
@@ -7457,7 +7457,7 @@
           <t>Ek numune</t>
         </is>
       </c>
-      <c r="C14" s="50" t="n"/>
+      <c r="C14" s="49" t="n"/>
       <c r="D14" s="6" t="inlineStr">
         <is>
           <t>2 saatlik kompozit</t>
@@ -7467,7 +7467,7 @@
       <c r="F14" s="6" t="n"/>
       <c r="G14" s="6" t="n"/>
       <c r="H14" s="6" t="n"/>
-      <c r="I14" s="25" t="n">
+      <c r="I14" s="22" t="n">
         <v>150</v>
       </c>
       <c r="J14" s="6">
@@ -7475,7 +7475,7 @@
         <v/>
       </c>
       <c r="K14" s="6" t="n"/>
-      <c r="L14" s="25" t="n">
+      <c r="L14" s="22" t="n">
         <v>200</v>
       </c>
       <c r="M14" s="6">
@@ -7483,10 +7483,10 @@
         <v/>
       </c>
       <c r="N14" s="6" t="n"/>
-      <c r="O14" s="25" t="n">
+      <c r="O14" s="22" t="n">
         <v>6</v>
       </c>
-      <c r="P14" s="25" t="n">
+      <c r="P14" s="22" t="n">
         <v>9</v>
       </c>
       <c r="Q14" s="6">
@@ -7501,7 +7501,7 @@
         <f>IF(R14="AŞIM","Evet",IF(R14="UYGUN","Hayır",""))</f>
         <v/>
       </c>
-      <c r="T14" s="50" t="n"/>
+      <c r="T14" s="49" t="n"/>
       <c r="U14" s="6" t="n"/>
       <c r="V14" s="6" t="n"/>
       <c r="W14" s="6" t="inlineStr">
@@ -7521,7 +7521,7 @@
           <t>Ek numune</t>
         </is>
       </c>
-      <c r="C15" s="50" t="n"/>
+      <c r="C15" s="49" t="n"/>
       <c r="D15" s="6" t="inlineStr">
         <is>
           <t>2 saatlik kompozit</t>
@@ -7531,7 +7531,7 @@
       <c r="F15" s="6" t="n"/>
       <c r="G15" s="6" t="n"/>
       <c r="H15" s="6" t="n"/>
-      <c r="I15" s="25" t="n">
+      <c r="I15" s="22" t="n">
         <v>150</v>
       </c>
       <c r="J15" s="6">
@@ -7539,7 +7539,7 @@
         <v/>
       </c>
       <c r="K15" s="6" t="n"/>
-      <c r="L15" s="25" t="n">
+      <c r="L15" s="22" t="n">
         <v>200</v>
       </c>
       <c r="M15" s="6">
@@ -7547,10 +7547,10 @@
         <v/>
       </c>
       <c r="N15" s="6" t="n"/>
-      <c r="O15" s="25" t="n">
+      <c r="O15" s="22" t="n">
         <v>6</v>
       </c>
-      <c r="P15" s="25" t="n">
+      <c r="P15" s="22" t="n">
         <v>9</v>
       </c>
       <c r="Q15" s="6">
@@ -7565,7 +7565,7 @@
         <f>IF(R15="AŞIM","Evet",IF(R15="UYGUN","Hayır",""))</f>
         <v/>
       </c>
-      <c r="T15" s="50" t="n"/>
+      <c r="T15" s="49" t="n"/>
       <c r="U15" s="6" t="n"/>
       <c r="V15" s="6" t="n"/>
       <c r="W15" s="6" t="inlineStr">
@@ -7585,7 +7585,7 @@
           <t>Ek numune</t>
         </is>
       </c>
-      <c r="C16" s="50" t="n"/>
+      <c r="C16" s="49" t="n"/>
       <c r="D16" s="6" t="inlineStr">
         <is>
           <t>2 saatlik kompozit</t>
@@ -7595,7 +7595,7 @@
       <c r="F16" s="6" t="n"/>
       <c r="G16" s="6" t="n"/>
       <c r="H16" s="6" t="n"/>
-      <c r="I16" s="25" t="n">
+      <c r="I16" s="22" t="n">
         <v>150</v>
       </c>
       <c r="J16" s="6">
@@ -7603,7 +7603,7 @@
         <v/>
       </c>
       <c r="K16" s="6" t="n"/>
-      <c r="L16" s="25" t="n">
+      <c r="L16" s="22" t="n">
         <v>200</v>
       </c>
       <c r="M16" s="6">
@@ -7611,10 +7611,10 @@
         <v/>
       </c>
       <c r="N16" s="6" t="n"/>
-      <c r="O16" s="25" t="n">
+      <c r="O16" s="22" t="n">
         <v>6</v>
       </c>
-      <c r="P16" s="25" t="n">
+      <c r="P16" s="22" t="n">
         <v>9</v>
       </c>
       <c r="Q16" s="6">
@@ -7629,7 +7629,7 @@
         <f>IF(R16="AŞIM","Evet",IF(R16="UYGUN","Hayır",""))</f>
         <v/>
       </c>
-      <c r="T16" s="50" t="n"/>
+      <c r="T16" s="49" t="n"/>
       <c r="U16" s="6" t="n"/>
       <c r="V16" s="6" t="n"/>
       <c r="W16" s="6" t="inlineStr">
@@ -7649,7 +7649,7 @@
           <t>Ek numune</t>
         </is>
       </c>
-      <c r="C17" s="50" t="n"/>
+      <c r="C17" s="49" t="n"/>
       <c r="D17" s="6" t="inlineStr">
         <is>
           <t>2 saatlik kompozit</t>
@@ -7659,7 +7659,7 @@
       <c r="F17" s="6" t="n"/>
       <c r="G17" s="6" t="n"/>
       <c r="H17" s="6" t="n"/>
-      <c r="I17" s="25" t="n">
+      <c r="I17" s="22" t="n">
         <v>150</v>
       </c>
       <c r="J17" s="6">
@@ -7667,7 +7667,7 @@
         <v/>
       </c>
       <c r="K17" s="6" t="n"/>
-      <c r="L17" s="25" t="n">
+      <c r="L17" s="22" t="n">
         <v>200</v>
       </c>
       <c r="M17" s="6">
@@ -7675,10 +7675,10 @@
         <v/>
       </c>
       <c r="N17" s="6" t="n"/>
-      <c r="O17" s="25" t="n">
+      <c r="O17" s="22" t="n">
         <v>6</v>
       </c>
-      <c r="P17" s="25" t="n">
+      <c r="P17" s="22" t="n">
         <v>9</v>
       </c>
       <c r="Q17" s="6">
@@ -7693,7 +7693,7 @@
         <f>IF(R17="AŞIM","Evet",IF(R17="UYGUN","Hayır",""))</f>
         <v/>
       </c>
-      <c r="T17" s="50" t="n"/>
+      <c r="T17" s="49" t="n"/>
       <c r="U17" s="6" t="n"/>
       <c r="V17" s="6" t="n"/>
       <c r="W17" s="6" t="inlineStr">
@@ -7895,7 +7895,7 @@
       </c>
     </row>
     <row r="5" ht="18" customHeight="1">
-      <c r="A5" s="50" t="n"/>
+      <c r="A5" s="49" t="n"/>
       <c r="B5" s="6" t="n"/>
       <c r="C5" s="6" t="n"/>
       <c r="D5" s="6" t="n"/>
@@ -7931,7 +7931,7 @@
       <c r="P6" s="18" t="n"/>
     </row>
     <row r="7" ht="18" customHeight="1">
-      <c r="A7" s="50" t="n"/>
+      <c r="A7" s="49" t="n"/>
       <c r="B7" s="6" t="n"/>
       <c r="C7" s="6" t="n"/>
       <c r="D7" s="6" t="n"/>
@@ -7967,7 +7967,7 @@
       <c r="P8" s="18" t="n"/>
     </row>
     <row r="9" ht="18" customHeight="1">
-      <c r="A9" s="50" t="n"/>
+      <c r="A9" s="49" t="n"/>
       <c r="B9" s="6" t="n"/>
       <c r="C9" s="6" t="n"/>
       <c r="D9" s="6" t="n"/>
@@ -8003,7 +8003,7 @@
       <c r="P10" s="18" t="n"/>
     </row>
     <row r="11" ht="18" customHeight="1">
-      <c r="A11" s="50" t="n"/>
+      <c r="A11" s="49" t="n"/>
       <c r="B11" s="6" t="n"/>
       <c r="C11" s="6" t="n"/>
       <c r="D11" s="6" t="n"/>
@@ -8039,7 +8039,7 @@
       <c r="P12" s="18" t="n"/>
     </row>
     <row r="13" ht="18" customHeight="1">
-      <c r="A13" s="50" t="n"/>
+      <c r="A13" s="49" t="n"/>
       <c r="B13" s="6" t="n"/>
       <c r="C13" s="6" t="n"/>
       <c r="D13" s="6" t="n"/>
@@ -8075,7 +8075,7 @@
       <c r="P14" s="18" t="n"/>
     </row>
     <row r="15" ht="18" customHeight="1">
-      <c r="A15" s="50" t="n"/>
+      <c r="A15" s="49" t="n"/>
       <c r="B15" s="6" t="n"/>
       <c r="C15" s="6" t="n"/>
       <c r="D15" s="6" t="n"/>
@@ -8111,7 +8111,7 @@
       <c r="P16" s="18" t="n"/>
     </row>
     <row r="17" ht="18" customHeight="1">
-      <c r="A17" s="50" t="n"/>
+      <c r="A17" s="49" t="n"/>
       <c r="B17" s="6" t="n"/>
       <c r="C17" s="6" t="n"/>
       <c r="D17" s="6" t="n"/>
@@ -8147,7 +8147,7 @@
       <c r="P18" s="18" t="n"/>
     </row>
     <row r="19" ht="18" customHeight="1">
-      <c r="A19" s="50" t="n"/>
+      <c r="A19" s="49" t="n"/>
       <c r="B19" s="6" t="n"/>
       <c r="C19" s="6" t="n"/>
       <c r="D19" s="6" t="n"/>
@@ -8183,7 +8183,7 @@
       <c r="P20" s="18" t="n"/>
     </row>
     <row r="21" ht="18" customHeight="1">
-      <c r="A21" s="50" t="n"/>
+      <c r="A21" s="49" t="n"/>
       <c r="B21" s="6" t="n"/>
       <c r="C21" s="6" t="n"/>
       <c r="D21" s="6" t="n"/>
@@ -8219,7 +8219,7 @@
       <c r="P22" s="18" t="n"/>
     </row>
     <row r="23" ht="18" customHeight="1">
-      <c r="A23" s="50" t="n"/>
+      <c r="A23" s="49" t="n"/>
       <c r="B23" s="6" t="n"/>
       <c r="C23" s="6" t="n"/>
       <c r="D23" s="6" t="n"/>
@@ -8255,7 +8255,7 @@
       <c r="P24" s="18" t="n"/>
     </row>
     <row r="25" ht="18" customHeight="1">
-      <c r="A25" s="50" t="n"/>
+      <c r="A25" s="49" t="n"/>
       <c r="B25" s="6" t="n"/>
       <c r="C25" s="6" t="n"/>
       <c r="D25" s="6" t="n"/>
@@ -8291,7 +8291,7 @@
       <c r="P26" s="18" t="n"/>
     </row>
     <row r="27" ht="18" customHeight="1">
-      <c r="A27" s="50" t="n"/>
+      <c r="A27" s="49" t="n"/>
       <c r="B27" s="6" t="n"/>
       <c r="C27" s="6" t="n"/>
       <c r="D27" s="6" t="n"/>
@@ -8327,7 +8327,7 @@
       <c r="P28" s="18" t="n"/>
     </row>
     <row r="29" ht="18" customHeight="1">
-      <c r="A29" s="50" t="n"/>
+      <c r="A29" s="49" t="n"/>
       <c r="B29" s="6" t="n"/>
       <c r="C29" s="6" t="n"/>
       <c r="D29" s="6" t="n"/>
@@ -8363,7 +8363,7 @@
       <c r="P30" s="18" t="n"/>
     </row>
     <row r="31" ht="18" customHeight="1">
-      <c r="A31" s="50" t="n"/>
+      <c r="A31" s="49" t="n"/>
       <c r="B31" s="6" t="n"/>
       <c r="C31" s="6" t="n"/>
       <c r="D31" s="6" t="n"/>
@@ -8399,7 +8399,7 @@
       <c r="P32" s="18" t="n"/>
     </row>
     <row r="33" ht="18" customHeight="1">
-      <c r="A33" s="50" t="n"/>
+      <c r="A33" s="49" t="n"/>
       <c r="B33" s="6" t="n"/>
       <c r="C33" s="6" t="n"/>
       <c r="D33" s="6" t="n"/>
@@ -8435,7 +8435,7 @@
       <c r="P34" s="18" t="n"/>
     </row>
     <row r="35" ht="18" customHeight="1">
-      <c r="A35" s="50" t="n"/>
+      <c r="A35" s="49" t="n"/>
       <c r="B35" s="6" t="n"/>
       <c r="C35" s="6" t="n"/>
       <c r="D35" s="6" t="n"/>
@@ -8471,7 +8471,7 @@
       <c r="P36" s="18" t="n"/>
     </row>
     <row r="37" ht="18" customHeight="1">
-      <c r="A37" s="50" t="n"/>
+      <c r="A37" s="49" t="n"/>
       <c r="B37" s="6" t="n"/>
       <c r="C37" s="6" t="n"/>
       <c r="D37" s="6" t="n"/>
@@ -8507,7 +8507,7 @@
       <c r="P38" s="18" t="n"/>
     </row>
     <row r="39" ht="18" customHeight="1">
-      <c r="A39" s="50" t="n"/>
+      <c r="A39" s="49" t="n"/>
       <c r="B39" s="6" t="n"/>
       <c r="C39" s="6" t="n"/>
       <c r="D39" s="6" t="n"/>
@@ -8543,7 +8543,7 @@
       <c r="P40" s="18" t="n"/>
     </row>
     <row r="41" ht="18" customHeight="1">
-      <c r="A41" s="50" t="n"/>
+      <c r="A41" s="49" t="n"/>
       <c r="B41" s="6" t="n"/>
       <c r="C41" s="6" t="n"/>
       <c r="D41" s="6" t="n"/>
@@ -8579,7 +8579,7 @@
       <c r="P42" s="18" t="n"/>
     </row>
     <row r="43" ht="18" customHeight="1">
-      <c r="A43" s="50" t="n"/>
+      <c r="A43" s="49" t="n"/>
       <c r="B43" s="6" t="n"/>
       <c r="C43" s="6" t="n"/>
       <c r="D43" s="6" t="n"/>
@@ -8615,7 +8615,7 @@
       <c r="P44" s="18" t="n"/>
     </row>
     <row r="45" ht="18" customHeight="1">
-      <c r="A45" s="50" t="n"/>
+      <c r="A45" s="49" t="n"/>
       <c r="B45" s="6" t="n"/>
       <c r="C45" s="6" t="n"/>
       <c r="D45" s="6" t="n"/>
@@ -8651,7 +8651,7 @@
       <c r="P46" s="18" t="n"/>
     </row>
     <row r="47" ht="18" customHeight="1">
-      <c r="A47" s="50" t="n"/>
+      <c r="A47" s="49" t="n"/>
       <c r="B47" s="6" t="n"/>
       <c r="C47" s="6" t="n"/>
       <c r="D47" s="6" t="n"/>
@@ -8687,7 +8687,7 @@
       <c r="P48" s="18" t="n"/>
     </row>
     <row r="49" ht="18" customHeight="1">
-      <c r="A49" s="50" t="n"/>
+      <c r="A49" s="49" t="n"/>
       <c r="B49" s="6" t="n"/>
       <c r="C49" s="6" t="n"/>
       <c r="D49" s="6" t="n"/>
@@ -8723,7 +8723,7 @@
       <c r="P50" s="18" t="n"/>
     </row>
     <row r="51" ht="18" customHeight="1">
-      <c r="A51" s="50" t="n"/>
+      <c r="A51" s="49" t="n"/>
       <c r="B51" s="6" t="n"/>
       <c r="C51" s="6" t="n"/>
       <c r="D51" s="6" t="n"/>
@@ -8759,7 +8759,7 @@
       <c r="P52" s="18" t="n"/>
     </row>
     <row r="53" ht="18" customHeight="1">
-      <c r="A53" s="50" t="n"/>
+      <c r="A53" s="49" t="n"/>
       <c r="B53" s="6" t="n"/>
       <c r="C53" s="6" t="n"/>
       <c r="D53" s="6" t="n"/>
@@ -8795,7 +8795,7 @@
       <c r="P54" s="18" t="n"/>
     </row>
     <row r="55" ht="18" customHeight="1">
-      <c r="A55" s="50" t="n"/>
+      <c r="A55" s="49" t="n"/>
       <c r="B55" s="6" t="n"/>
       <c r="C55" s="6" t="n"/>
       <c r="D55" s="6" t="n"/>
@@ -8831,7 +8831,7 @@
       <c r="P56" s="18" t="n"/>
     </row>
     <row r="57" ht="18" customHeight="1">
-      <c r="A57" s="50" t="n"/>
+      <c r="A57" s="49" t="n"/>
       <c r="B57" s="6" t="n"/>
       <c r="C57" s="6" t="n"/>
       <c r="D57" s="6" t="n"/>
@@ -8867,7 +8867,7 @@
       <c r="P58" s="18" t="n"/>
     </row>
     <row r="59" ht="18" customHeight="1">
-      <c r="A59" s="50" t="n"/>
+      <c r="A59" s="49" t="n"/>
       <c r="B59" s="6" t="n"/>
       <c r="C59" s="6" t="n"/>
       <c r="D59" s="6" t="n"/>
@@ -8903,7 +8903,7 @@
       <c r="P60" s="18" t="n"/>
     </row>
     <row r="61" ht="18" customHeight="1">
-      <c r="A61" s="50" t="n"/>
+      <c r="A61" s="49" t="n"/>
       <c r="B61" s="6" t="n"/>
       <c r="C61" s="6" t="n"/>
       <c r="D61" s="6" t="n"/>
@@ -8939,7 +8939,7 @@
       <c r="P62" s="18" t="n"/>
     </row>
     <row r="63" ht="18" customHeight="1">
-      <c r="A63" s="50" t="n"/>
+      <c r="A63" s="49" t="n"/>
       <c r="B63" s="6" t="n"/>
       <c r="C63" s="6" t="n"/>
       <c r="D63" s="6" t="n"/>
@@ -8975,7 +8975,7 @@
       <c r="P64" s="18" t="n"/>
     </row>
     <row r="65" ht="18" customHeight="1">
-      <c r="A65" s="50" t="n"/>
+      <c r="A65" s="49" t="n"/>
       <c r="B65" s="6" t="n"/>
       <c r="C65" s="6" t="n"/>
       <c r="D65" s="6" t="n"/>
@@ -9011,7 +9011,7 @@
       <c r="P66" s="18" t="n"/>
     </row>
     <row r="67" ht="18" customHeight="1">
-      <c r="A67" s="50" t="n"/>
+      <c r="A67" s="49" t="n"/>
       <c r="B67" s="6" t="n"/>
       <c r="C67" s="6" t="n"/>
       <c r="D67" s="6" t="n"/>
@@ -9047,7 +9047,7 @@
       <c r="P68" s="18" t="n"/>
     </row>
     <row r="69" ht="18" customHeight="1">
-      <c r="A69" s="50" t="n"/>
+      <c r="A69" s="49" t="n"/>
       <c r="B69" s="6" t="n"/>
       <c r="C69" s="6" t="n"/>
       <c r="D69" s="6" t="n"/>
@@ -9083,7 +9083,7 @@
       <c r="P70" s="18" t="n"/>
     </row>
     <row r="71" ht="18" customHeight="1">
-      <c r="A71" s="50" t="n"/>
+      <c r="A71" s="49" t="n"/>
       <c r="B71" s="6" t="n"/>
       <c r="C71" s="6" t="n"/>
       <c r="D71" s="6" t="n"/>
@@ -9119,7 +9119,7 @@
       <c r="P72" s="18" t="n"/>
     </row>
     <row r="73" ht="18" customHeight="1">
-      <c r="A73" s="50" t="n"/>
+      <c r="A73" s="49" t="n"/>
       <c r="B73" s="6" t="n"/>
       <c r="C73" s="6" t="n"/>
       <c r="D73" s="6" t="n"/>
@@ -9155,7 +9155,7 @@
       <c r="P74" s="18" t="n"/>
     </row>
     <row r="75" ht="18" customHeight="1">
-      <c r="A75" s="50" t="n"/>
+      <c r="A75" s="49" t="n"/>
       <c r="B75" s="6" t="n"/>
       <c r="C75" s="6" t="n"/>
       <c r="D75" s="6" t="n"/>
@@ -9191,7 +9191,7 @@
       <c r="P76" s="18" t="n"/>
     </row>
     <row r="77" ht="18" customHeight="1">
-      <c r="A77" s="50" t="n"/>
+      <c r="A77" s="49" t="n"/>
       <c r="B77" s="6" t="n"/>
       <c r="C77" s="6" t="n"/>
       <c r="D77" s="6" t="n"/>
@@ -9227,7 +9227,7 @@
       <c r="P78" s="18" t="n"/>
     </row>
     <row r="79" ht="18" customHeight="1">
-      <c r="A79" s="50" t="n"/>
+      <c r="A79" s="49" t="n"/>
       <c r="B79" s="6" t="n"/>
       <c r="C79" s="6" t="n"/>
       <c r="D79" s="6" t="n"/>
@@ -9263,7 +9263,7 @@
       <c r="P80" s="18" t="n"/>
     </row>
     <row r="81" ht="18" customHeight="1">
-      <c r="A81" s="50" t="n"/>
+      <c r="A81" s="49" t="n"/>
       <c r="B81" s="6" t="n"/>
       <c r="C81" s="6" t="n"/>
       <c r="D81" s="6" t="n"/>
@@ -9299,7 +9299,7 @@
       <c r="P82" s="18" t="n"/>
     </row>
     <row r="83" ht="18" customHeight="1">
-      <c r="A83" s="50" t="n"/>
+      <c r="A83" s="49" t="n"/>
       <c r="B83" s="6" t="n"/>
       <c r="C83" s="6" t="n"/>
       <c r="D83" s="6" t="n"/>
@@ -9335,7 +9335,7 @@
       <c r="P84" s="18" t="n"/>
     </row>
     <row r="85" ht="18" customHeight="1">
-      <c r="A85" s="50" t="n"/>
+      <c r="A85" s="49" t="n"/>
       <c r="B85" s="6" t="n"/>
       <c r="C85" s="6" t="n"/>
       <c r="D85" s="6" t="n"/>
@@ -9371,7 +9371,7 @@
       <c r="P86" s="18" t="n"/>
     </row>
     <row r="87" ht="18" customHeight="1">
-      <c r="A87" s="50" t="n"/>
+      <c r="A87" s="49" t="n"/>
       <c r="B87" s="6" t="n"/>
       <c r="C87" s="6" t="n"/>
       <c r="D87" s="6" t="n"/>
@@ -9407,7 +9407,7 @@
       <c r="P88" s="18" t="n"/>
     </row>
     <row r="89" ht="18" customHeight="1">
-      <c r="A89" s="50" t="n"/>
+      <c r="A89" s="49" t="n"/>
       <c r="B89" s="6" t="n"/>
       <c r="C89" s="6" t="n"/>
       <c r="D89" s="6" t="n"/>
@@ -9443,7 +9443,7 @@
       <c r="P90" s="18" t="n"/>
     </row>
     <row r="91" ht="18" customHeight="1">
-      <c r="A91" s="50" t="n"/>
+      <c r="A91" s="49" t="n"/>
       <c r="B91" s="6" t="n"/>
       <c r="C91" s="6" t="n"/>
       <c r="D91" s="6" t="n"/>
@@ -9479,7 +9479,7 @@
       <c r="P92" s="18" t="n"/>
     </row>
     <row r="93" ht="18" customHeight="1">
-      <c r="A93" s="50" t="n"/>
+      <c r="A93" s="49" t="n"/>
       <c r="B93" s="6" t="n"/>
       <c r="C93" s="6" t="n"/>
       <c r="D93" s="6" t="n"/>
@@ -9515,7 +9515,7 @@
       <c r="P94" s="18" t="n"/>
     </row>
     <row r="95" ht="18" customHeight="1">
-      <c r="A95" s="50" t="n"/>
+      <c r="A95" s="49" t="n"/>
       <c r="B95" s="6" t="n"/>
       <c r="C95" s="6" t="n"/>
       <c r="D95" s="6" t="n"/>
@@ -9551,7 +9551,7 @@
       <c r="P96" s="18" t="n"/>
     </row>
     <row r="97" ht="18" customHeight="1">
-      <c r="A97" s="50" t="n"/>
+      <c r="A97" s="49" t="n"/>
       <c r="B97" s="6" t="n"/>
       <c r="C97" s="6" t="n"/>
       <c r="D97" s="6" t="n"/>
@@ -9587,7 +9587,7 @@
       <c r="P98" s="18" t="n"/>
     </row>
     <row r="99" ht="18" customHeight="1">
-      <c r="A99" s="50" t="n"/>
+      <c r="A99" s="49" t="n"/>
       <c r="B99" s="6" t="n"/>
       <c r="C99" s="6" t="n"/>
       <c r="D99" s="6" t="n"/>
@@ -9623,7 +9623,7 @@
       <c r="P100" s="18" t="n"/>
     </row>
     <row r="101" ht="18" customHeight="1">
-      <c r="A101" s="50" t="n"/>
+      <c r="A101" s="49" t="n"/>
       <c r="B101" s="6" t="n"/>
       <c r="C101" s="6" t="n"/>
       <c r="D101" s="6" t="n"/>
@@ -9659,7 +9659,7 @@
       <c r="P102" s="18" t="n"/>
     </row>
     <row r="103" ht="18" customHeight="1">
-      <c r="A103" s="50" t="n"/>
+      <c r="A103" s="49" t="n"/>
       <c r="B103" s="6" t="n"/>
       <c r="C103" s="6" t="n"/>
       <c r="D103" s="6" t="n"/>
@@ -9695,7 +9695,7 @@
       <c r="P104" s="18" t="n"/>
     </row>
     <row r="105" ht="18" customHeight="1">
-      <c r="A105" s="50" t="n"/>
+      <c r="A105" s="49" t="n"/>
       <c r="B105" s="6" t="n"/>
       <c r="C105" s="6" t="n"/>
       <c r="D105" s="6" t="n"/>
@@ -9731,7 +9731,7 @@
       <c r="P106" s="18" t="n"/>
     </row>
     <row r="107" ht="18" customHeight="1">
-      <c r="A107" s="50" t="n"/>
+      <c r="A107" s="49" t="n"/>
       <c r="B107" s="6" t="n"/>
       <c r="C107" s="6" t="n"/>
       <c r="D107" s="6" t="n"/>
@@ -9767,7 +9767,7 @@
       <c r="P108" s="18" t="n"/>
     </row>
     <row r="109" ht="18" customHeight="1">
-      <c r="A109" s="50" t="n"/>
+      <c r="A109" s="49" t="n"/>
       <c r="B109" s="6" t="n"/>
       <c r="C109" s="6" t="n"/>
       <c r="D109" s="6" t="n"/>
@@ -9803,7 +9803,7 @@
       <c r="P110" s="18" t="n"/>
     </row>
     <row r="111" ht="18" customHeight="1">
-      <c r="A111" s="50" t="n"/>
+      <c r="A111" s="49" t="n"/>
       <c r="B111" s="6" t="n"/>
       <c r="C111" s="6" t="n"/>
       <c r="D111" s="6" t="n"/>
@@ -9839,7 +9839,7 @@
       <c r="P112" s="18" t="n"/>
     </row>
     <row r="113" ht="18" customHeight="1">
-      <c r="A113" s="50" t="n"/>
+      <c r="A113" s="49" t="n"/>
       <c r="B113" s="6" t="n"/>
       <c r="C113" s="6" t="n"/>
       <c r="D113" s="6" t="n"/>
@@ -9875,7 +9875,7 @@
       <c r="P114" s="18" t="n"/>
     </row>
     <row r="115" ht="18" customHeight="1">
-      <c r="A115" s="50" t="n"/>
+      <c r="A115" s="49" t="n"/>
       <c r="B115" s="6" t="n"/>
       <c r="C115" s="6" t="n"/>
       <c r="D115" s="6" t="n"/>
@@ -9911,7 +9911,7 @@
       <c r="P116" s="18" t="n"/>
     </row>
     <row r="117" ht="18" customHeight="1">
-      <c r="A117" s="50" t="n"/>
+      <c r="A117" s="49" t="n"/>
       <c r="B117" s="6" t="n"/>
       <c r="C117" s="6" t="n"/>
       <c r="D117" s="6" t="n"/>
@@ -9947,7 +9947,7 @@
       <c r="P118" s="18" t="n"/>
     </row>
     <row r="119" ht="18" customHeight="1">
-      <c r="A119" s="50" t="n"/>
+      <c r="A119" s="49" t="n"/>
       <c r="B119" s="6" t="n"/>
       <c r="C119" s="6" t="n"/>
       <c r="D119" s="6" t="n"/>
@@ -9983,7 +9983,7 @@
       <c r="P120" s="18" t="n"/>
     </row>
     <row r="121" ht="18" customHeight="1">
-      <c r="A121" s="50" t="n"/>
+      <c r="A121" s="49" t="n"/>
       <c r="B121" s="6" t="n"/>
       <c r="C121" s="6" t="n"/>
       <c r="D121" s="6" t="n"/>
@@ -10019,7 +10019,7 @@
       <c r="P122" s="18" t="n"/>
     </row>
     <row r="123" ht="18" customHeight="1">
-      <c r="A123" s="50" t="n"/>
+      <c r="A123" s="49" t="n"/>
       <c r="B123" s="6" t="n"/>
       <c r="C123" s="6" t="n"/>
       <c r="D123" s="6" t="n"/>
@@ -10203,7 +10203,7 @@
       </c>
       <c r="B5" s="6" t="n"/>
       <c r="C5" s="6" t="n"/>
-      <c r="D5" s="25">
+      <c r="D5" s="22">
         <f>IF(COUNT(B5,C5)=0,"",N(B5)+N(C5))</f>
         <v/>
       </c>
@@ -10211,7 +10211,7 @@
       <c r="F5" s="6" t="n"/>
       <c r="G5" s="6" t="n"/>
       <c r="H5" s="6" t="n"/>
-      <c r="I5" s="25">
+      <c r="I5" s="22">
         <f>IF(OR(D5="",H5=""),"",D5-H5)</f>
         <v/>
       </c>
@@ -10227,7 +10227,7 @@
       </c>
       <c r="B6" s="18" t="n"/>
       <c r="C6" s="18" t="n"/>
-      <c r="D6" s="25">
+      <c r="D6" s="22">
         <f>IF(COUNT(B6,C6)=0,"",N(B6)+N(C6))</f>
         <v/>
       </c>
@@ -10235,7 +10235,7 @@
       <c r="F6" s="18" t="n"/>
       <c r="G6" s="18" t="n"/>
       <c r="H6" s="18" t="n"/>
-      <c r="I6" s="25">
+      <c r="I6" s="22">
         <f>IF(OR(D6="",H6=""),"",D6-H6)</f>
         <v/>
       </c>
@@ -10251,7 +10251,7 @@
       </c>
       <c r="B7" s="6" t="n"/>
       <c r="C7" s="6" t="n"/>
-      <c r="D7" s="25">
+      <c r="D7" s="22">
         <f>IF(COUNT(B7,C7)=0,"",N(B7)+N(C7))</f>
         <v/>
       </c>
@@ -10259,7 +10259,7 @@
       <c r="F7" s="6" t="n"/>
       <c r="G7" s="6" t="n"/>
       <c r="H7" s="6" t="n"/>
-      <c r="I7" s="25">
+      <c r="I7" s="22">
         <f>IF(OR(D7="",H7=""),"",D7-H7)</f>
         <v/>
       </c>
@@ -10275,7 +10275,7 @@
       </c>
       <c r="B8" s="18" t="n"/>
       <c r="C8" s="18" t="n"/>
-      <c r="D8" s="25">
+      <c r="D8" s="22">
         <f>IF(COUNT(B8,C8)=0,"",N(B8)+N(C8))</f>
         <v/>
       </c>
@@ -10283,7 +10283,7 @@
       <c r="F8" s="18" t="n"/>
       <c r="G8" s="18" t="n"/>
       <c r="H8" s="18" t="n"/>
-      <c r="I8" s="25">
+      <c r="I8" s="22">
         <f>IF(OR(D8="",H8=""),"",D8-H8)</f>
         <v/>
       </c>
@@ -10299,7 +10299,7 @@
       </c>
       <c r="B9" s="6" t="n"/>
       <c r="C9" s="6" t="n"/>
-      <c r="D9" s="25">
+      <c r="D9" s="22">
         <f>IF(COUNT(B9,C9)=0,"",N(B9)+N(C9))</f>
         <v/>
       </c>
@@ -10307,7 +10307,7 @@
       <c r="F9" s="6" t="n"/>
       <c r="G9" s="6" t="n"/>
       <c r="H9" s="6" t="n"/>
-      <c r="I9" s="25">
+      <c r="I9" s="22">
         <f>IF(OR(D9="",H9=""),"",D9-H9)</f>
         <v/>
       </c>
@@ -10323,7 +10323,7 @@
       </c>
       <c r="B10" s="18" t="n"/>
       <c r="C10" s="18" t="n"/>
-      <c r="D10" s="25">
+      <c r="D10" s="22">
         <f>IF(COUNT(B10,C10)=0,"",N(B10)+N(C10))</f>
         <v/>
       </c>
@@ -10331,7 +10331,7 @@
       <c r="F10" s="18" t="n"/>
       <c r="G10" s="18" t="n"/>
       <c r="H10" s="18" t="n"/>
-      <c r="I10" s="25">
+      <c r="I10" s="22">
         <f>IF(OR(D10="",H10=""),"",D10-H10)</f>
         <v/>
       </c>
@@ -10347,7 +10347,7 @@
       </c>
       <c r="B11" s="6" t="n"/>
       <c r="C11" s="6" t="n"/>
-      <c r="D11" s="25">
+      <c r="D11" s="22">
         <f>IF(COUNT(B11,C11)=0,"",N(B11)+N(C11))</f>
         <v/>
       </c>
@@ -10355,7 +10355,7 @@
       <c r="F11" s="6" t="n"/>
       <c r="G11" s="6" t="n"/>
       <c r="H11" s="6" t="n"/>
-      <c r="I11" s="25">
+      <c r="I11" s="22">
         <f>IF(OR(D11="",H11=""),"",D11-H11)</f>
         <v/>
       </c>
@@ -10371,7 +10371,7 @@
       </c>
       <c r="B12" s="18" t="n"/>
       <c r="C12" s="18" t="n"/>
-      <c r="D12" s="25">
+      <c r="D12" s="22">
         <f>IF(COUNT(B12,C12)=0,"",N(B12)+N(C12))</f>
         <v/>
       </c>
@@ -10379,7 +10379,7 @@
       <c r="F12" s="18" t="n"/>
       <c r="G12" s="18" t="n"/>
       <c r="H12" s="18" t="n"/>
-      <c r="I12" s="25">
+      <c r="I12" s="22">
         <f>IF(OR(D12="",H12=""),"",D12-H12)</f>
         <v/>
       </c>
@@ -10395,7 +10395,7 @@
       </c>
       <c r="B13" s="6" t="n"/>
       <c r="C13" s="6" t="n"/>
-      <c r="D13" s="25">
+      <c r="D13" s="22">
         <f>IF(COUNT(B13,C13)=0,"",N(B13)+N(C13))</f>
         <v/>
       </c>
@@ -10403,7 +10403,7 @@
       <c r="F13" s="6" t="n"/>
       <c r="G13" s="6" t="n"/>
       <c r="H13" s="6" t="n"/>
-      <c r="I13" s="25">
+      <c r="I13" s="22">
         <f>IF(OR(D13="",H13=""),"",D13-H13)</f>
         <v/>
       </c>
@@ -10419,7 +10419,7 @@
       </c>
       <c r="B14" s="18" t="n"/>
       <c r="C14" s="18" t="n"/>
-      <c r="D14" s="25">
+      <c r="D14" s="22">
         <f>IF(COUNT(B14,C14)=0,"",N(B14)+N(C14))</f>
         <v/>
       </c>
@@ -10427,7 +10427,7 @@
       <c r="F14" s="18" t="n"/>
       <c r="G14" s="18" t="n"/>
       <c r="H14" s="18" t="n"/>
-      <c r="I14" s="25">
+      <c r="I14" s="22">
         <f>IF(OR(D14="",H14=""),"",D14-H14)</f>
         <v/>
       </c>
@@ -10443,7 +10443,7 @@
       </c>
       <c r="B15" s="6" t="n"/>
       <c r="C15" s="6" t="n"/>
-      <c r="D15" s="25">
+      <c r="D15" s="22">
         <f>IF(COUNT(B15,C15)=0,"",N(B15)+N(C15))</f>
         <v/>
       </c>
@@ -10451,7 +10451,7 @@
       <c r="F15" s="6" t="n"/>
       <c r="G15" s="6" t="n"/>
       <c r="H15" s="6" t="n"/>
-      <c r="I15" s="25">
+      <c r="I15" s="22">
         <f>IF(OR(D15="",H15=""),"",D15-H15)</f>
         <v/>
       </c>
@@ -10467,7 +10467,7 @@
       </c>
       <c r="B16" s="18" t="n"/>
       <c r="C16" s="18" t="n"/>
-      <c r="D16" s="25">
+      <c r="D16" s="22">
         <f>IF(COUNT(B16,C16)=0,"",N(B16)+N(C16))</f>
         <v/>
       </c>
@@ -10475,7 +10475,7 @@
       <c r="F16" s="18" t="n"/>
       <c r="G16" s="18" t="n"/>
       <c r="H16" s="18" t="n"/>
-      <c r="I16" s="25">
+      <c r="I16" s="22">
         <f>IF(OR(D16="",H16=""),"",D16-H16)</f>
         <v/>
       </c>
@@ -11040,7 +11040,7 @@
       </c>
     </row>
     <row r="20" ht="18" customHeight="1">
-      <c r="A20" s="50" t="n"/>
+      <c r="A20" s="49" t="n"/>
       <c r="B20" s="6" t="n"/>
       <c r="C20" s="6" t="n"/>
       <c r="D20" s="6" t="n"/>
@@ -11049,12 +11049,12 @@
       <c r="G20" s="6" t="n"/>
       <c r="H20" s="6" t="n"/>
       <c r="I20" s="6" t="n"/>
-      <c r="J20" s="50" t="n"/>
+      <c r="J20" s="49" t="n"/>
       <c r="K20" s="6" t="n"/>
       <c r="L20" s="6" t="n"/>
     </row>
     <row r="21" ht="18" customHeight="1">
-      <c r="A21" s="50" t="n"/>
+      <c r="A21" s="49" t="n"/>
       <c r="B21" s="6" t="n"/>
       <c r="C21" s="6" t="n"/>
       <c r="D21" s="6" t="n"/>
@@ -11063,12 +11063,12 @@
       <c r="G21" s="6" t="n"/>
       <c r="H21" s="6" t="n"/>
       <c r="I21" s="6" t="n"/>
-      <c r="J21" s="50" t="n"/>
+      <c r="J21" s="49" t="n"/>
       <c r="K21" s="6" t="n"/>
       <c r="L21" s="6" t="n"/>
     </row>
     <row r="22" ht="18" customHeight="1">
-      <c r="A22" s="50" t="n"/>
+      <c r="A22" s="49" t="n"/>
       <c r="B22" s="6" t="n"/>
       <c r="C22" s="6" t="n"/>
       <c r="D22" s="6" t="n"/>
@@ -11077,12 +11077,12 @@
       <c r="G22" s="6" t="n"/>
       <c r="H22" s="6" t="n"/>
       <c r="I22" s="6" t="n"/>
-      <c r="J22" s="50" t="n"/>
+      <c r="J22" s="49" t="n"/>
       <c r="K22" s="6" t="n"/>
       <c r="L22" s="6" t="n"/>
     </row>
     <row r="23" ht="18" customHeight="1">
-      <c r="A23" s="50" t="n"/>
+      <c r="A23" s="49" t="n"/>
       <c r="B23" s="6" t="n"/>
       <c r="C23" s="6" t="n"/>
       <c r="D23" s="6" t="n"/>
@@ -11091,12 +11091,12 @@
       <c r="G23" s="6" t="n"/>
       <c r="H23" s="6" t="n"/>
       <c r="I23" s="6" t="n"/>
-      <c r="J23" s="50" t="n"/>
+      <c r="J23" s="49" t="n"/>
       <c r="K23" s="6" t="n"/>
       <c r="L23" s="6" t="n"/>
     </row>
     <row r="24" ht="18" customHeight="1">
-      <c r="A24" s="50" t="n"/>
+      <c r="A24" s="49" t="n"/>
       <c r="B24" s="6" t="n"/>
       <c r="C24" s="6" t="n"/>
       <c r="D24" s="6" t="n"/>
@@ -11105,12 +11105,12 @@
       <c r="G24" s="6" t="n"/>
       <c r="H24" s="6" t="n"/>
       <c r="I24" s="6" t="n"/>
-      <c r="J24" s="50" t="n"/>
+      <c r="J24" s="49" t="n"/>
       <c r="K24" s="6" t="n"/>
       <c r="L24" s="6" t="n"/>
     </row>
     <row r="25" ht="18" customHeight="1">
-      <c r="A25" s="50" t="n"/>
+      <c r="A25" s="49" t="n"/>
       <c r="B25" s="6" t="n"/>
       <c r="C25" s="6" t="n"/>
       <c r="D25" s="6" t="n"/>
@@ -11119,12 +11119,12 @@
       <c r="G25" s="6" t="n"/>
       <c r="H25" s="6" t="n"/>
       <c r="I25" s="6" t="n"/>
-      <c r="J25" s="50" t="n"/>
+      <c r="J25" s="49" t="n"/>
       <c r="K25" s="6" t="n"/>
       <c r="L25" s="6" t="n"/>
     </row>
     <row r="26" ht="18" customHeight="1">
-      <c r="A26" s="50" t="n"/>
+      <c r="A26" s="49" t="n"/>
       <c r="B26" s="6" t="n"/>
       <c r="C26" s="6" t="n"/>
       <c r="D26" s="6" t="n"/>
@@ -11133,12 +11133,12 @@
       <c r="G26" s="6" t="n"/>
       <c r="H26" s="6" t="n"/>
       <c r="I26" s="6" t="n"/>
-      <c r="J26" s="50" t="n"/>
+      <c r="J26" s="49" t="n"/>
       <c r="K26" s="6" t="n"/>
       <c r="L26" s="6" t="n"/>
     </row>
     <row r="27" ht="18" customHeight="1">
-      <c r="A27" s="50" t="n"/>
+      <c r="A27" s="49" t="n"/>
       <c r="B27" s="6" t="n"/>
       <c r="C27" s="6" t="n"/>
       <c r="D27" s="6" t="n"/>
@@ -11147,12 +11147,12 @@
       <c r="G27" s="6" t="n"/>
       <c r="H27" s="6" t="n"/>
       <c r="I27" s="6" t="n"/>
-      <c r="J27" s="50" t="n"/>
+      <c r="J27" s="49" t="n"/>
       <c r="K27" s="6" t="n"/>
       <c r="L27" s="6" t="n"/>
     </row>
     <row r="28" ht="18" customHeight="1">
-      <c r="A28" s="50" t="n"/>
+      <c r="A28" s="49" t="n"/>
       <c r="B28" s="6" t="n"/>
       <c r="C28" s="6" t="n"/>
       <c r="D28" s="6" t="n"/>
@@ -11161,12 +11161,12 @@
       <c r="G28" s="6" t="n"/>
       <c r="H28" s="6" t="n"/>
       <c r="I28" s="6" t="n"/>
-      <c r="J28" s="50" t="n"/>
+      <c r="J28" s="49" t="n"/>
       <c r="K28" s="6" t="n"/>
       <c r="L28" s="6" t="n"/>
     </row>
     <row r="29" ht="18" customHeight="1">
-      <c r="A29" s="50" t="n"/>
+      <c r="A29" s="49" t="n"/>
       <c r="B29" s="6" t="n"/>
       <c r="C29" s="6" t="n"/>
       <c r="D29" s="6" t="n"/>
@@ -11175,12 +11175,12 @@
       <c r="G29" s="6" t="n"/>
       <c r="H29" s="6" t="n"/>
       <c r="I29" s="6" t="n"/>
-      <c r="J29" s="50" t="n"/>
+      <c r="J29" s="49" t="n"/>
       <c r="K29" s="6" t="n"/>
       <c r="L29" s="6" t="n"/>
     </row>
     <row r="30" ht="18" customHeight="1">
-      <c r="A30" s="50" t="n"/>
+      <c r="A30" s="49" t="n"/>
       <c r="B30" s="6" t="n"/>
       <c r="C30" s="6" t="n"/>
       <c r="D30" s="6" t="n"/>
@@ -11189,12 +11189,12 @@
       <c r="G30" s="6" t="n"/>
       <c r="H30" s="6" t="n"/>
       <c r="I30" s="6" t="n"/>
-      <c r="J30" s="50" t="n"/>
+      <c r="J30" s="49" t="n"/>
       <c r="K30" s="6" t="n"/>
       <c r="L30" s="6" t="n"/>
     </row>
     <row r="31" ht="18" customHeight="1">
-      <c r="A31" s="50" t="n"/>
+      <c r="A31" s="49" t="n"/>
       <c r="B31" s="6" t="n"/>
       <c r="C31" s="6" t="n"/>
       <c r="D31" s="6" t="n"/>
@@ -11203,12 +11203,12 @@
       <c r="G31" s="6" t="n"/>
       <c r="H31" s="6" t="n"/>
       <c r="I31" s="6" t="n"/>
-      <c r="J31" s="50" t="n"/>
+      <c r="J31" s="49" t="n"/>
       <c r="K31" s="6" t="n"/>
       <c r="L31" s="6" t="n"/>
     </row>
     <row r="32" ht="18" customHeight="1">
-      <c r="A32" s="50" t="n"/>
+      <c r="A32" s="49" t="n"/>
       <c r="B32" s="6" t="n"/>
       <c r="C32" s="6" t="n"/>
       <c r="D32" s="6" t="n"/>
@@ -11217,12 +11217,12 @@
       <c r="G32" s="6" t="n"/>
       <c r="H32" s="6" t="n"/>
       <c r="I32" s="6" t="n"/>
-      <c r="J32" s="50" t="n"/>
+      <c r="J32" s="49" t="n"/>
       <c r="K32" s="6" t="n"/>
       <c r="L32" s="6" t="n"/>
     </row>
     <row r="33" ht="18" customHeight="1">
-      <c r="A33" s="50" t="n"/>
+      <c r="A33" s="49" t="n"/>
       <c r="B33" s="6" t="n"/>
       <c r="C33" s="6" t="n"/>
       <c r="D33" s="6" t="n"/>
@@ -11231,12 +11231,12 @@
       <c r="G33" s="6" t="n"/>
       <c r="H33" s="6" t="n"/>
       <c r="I33" s="6" t="n"/>
-      <c r="J33" s="50" t="n"/>
+      <c r="J33" s="49" t="n"/>
       <c r="K33" s="6" t="n"/>
       <c r="L33" s="6" t="n"/>
     </row>
     <row r="34" ht="18" customHeight="1">
-      <c r="A34" s="50" t="n"/>
+      <c r="A34" s="49" t="n"/>
       <c r="B34" s="6" t="n"/>
       <c r="C34" s="6" t="n"/>
       <c r="D34" s="6" t="n"/>
@@ -11245,12 +11245,12 @@
       <c r="G34" s="6" t="n"/>
       <c r="H34" s="6" t="n"/>
       <c r="I34" s="6" t="n"/>
-      <c r="J34" s="50" t="n"/>
+      <c r="J34" s="49" t="n"/>
       <c r="K34" s="6" t="n"/>
       <c r="L34" s="6" t="n"/>
     </row>
     <row r="35" ht="18" customHeight="1">
-      <c r="A35" s="50" t="n"/>
+      <c r="A35" s="49" t="n"/>
       <c r="B35" s="6" t="n"/>
       <c r="C35" s="6" t="n"/>
       <c r="D35" s="6" t="n"/>
@@ -11259,12 +11259,12 @@
       <c r="G35" s="6" t="n"/>
       <c r="H35" s="6" t="n"/>
       <c r="I35" s="6" t="n"/>
-      <c r="J35" s="50" t="n"/>
+      <c r="J35" s="49" t="n"/>
       <c r="K35" s="6" t="n"/>
       <c r="L35" s="6" t="n"/>
     </row>
     <row r="36" ht="18" customHeight="1">
-      <c r="A36" s="50" t="n"/>
+      <c r="A36" s="49" t="n"/>
       <c r="B36" s="6" t="n"/>
       <c r="C36" s="6" t="n"/>
       <c r="D36" s="6" t="n"/>
@@ -11273,12 +11273,12 @@
       <c r="G36" s="6" t="n"/>
       <c r="H36" s="6" t="n"/>
       <c r="I36" s="6" t="n"/>
-      <c r="J36" s="50" t="n"/>
+      <c r="J36" s="49" t="n"/>
       <c r="K36" s="6" t="n"/>
       <c r="L36" s="6" t="n"/>
     </row>
     <row r="37" ht="18" customHeight="1">
-      <c r="A37" s="50" t="n"/>
+      <c r="A37" s="49" t="n"/>
       <c r="B37" s="6" t="n"/>
       <c r="C37" s="6" t="n"/>
       <c r="D37" s="6" t="n"/>
@@ -11287,12 +11287,12 @@
       <c r="G37" s="6" t="n"/>
       <c r="H37" s="6" t="n"/>
       <c r="I37" s="6" t="n"/>
-      <c r="J37" s="50" t="n"/>
+      <c r="J37" s="49" t="n"/>
       <c r="K37" s="6" t="n"/>
       <c r="L37" s="6" t="n"/>
     </row>
     <row r="38" ht="18" customHeight="1">
-      <c r="A38" s="50" t="n"/>
+      <c r="A38" s="49" t="n"/>
       <c r="B38" s="6" t="n"/>
       <c r="C38" s="6" t="n"/>
       <c r="D38" s="6" t="n"/>
@@ -11301,12 +11301,12 @@
       <c r="G38" s="6" t="n"/>
       <c r="H38" s="6" t="n"/>
       <c r="I38" s="6" t="n"/>
-      <c r="J38" s="50" t="n"/>
+      <c r="J38" s="49" t="n"/>
       <c r="K38" s="6" t="n"/>
       <c r="L38" s="6" t="n"/>
     </row>
     <row r="39" ht="18" customHeight="1">
-      <c r="A39" s="50" t="n"/>
+      <c r="A39" s="49" t="n"/>
       <c r="B39" s="6" t="n"/>
       <c r="C39" s="6" t="n"/>
       <c r="D39" s="6" t="n"/>
@@ -11315,12 +11315,12 @@
       <c r="G39" s="6" t="n"/>
       <c r="H39" s="6" t="n"/>
       <c r="I39" s="6" t="n"/>
-      <c r="J39" s="50" t="n"/>
+      <c r="J39" s="49" t="n"/>
       <c r="K39" s="6" t="n"/>
       <c r="L39" s="6" t="n"/>
     </row>
     <row r="40" ht="18" customHeight="1">
-      <c r="A40" s="50" t="n"/>
+      <c r="A40" s="49" t="n"/>
       <c r="B40" s="6" t="n"/>
       <c r="C40" s="6" t="n"/>
       <c r="D40" s="6" t="n"/>
@@ -11329,12 +11329,12 @@
       <c r="G40" s="6" t="n"/>
       <c r="H40" s="6" t="n"/>
       <c r="I40" s="6" t="n"/>
-      <c r="J40" s="50" t="n"/>
+      <c r="J40" s="49" t="n"/>
       <c r="K40" s="6" t="n"/>
       <c r="L40" s="6" t="n"/>
     </row>
     <row r="41" ht="18" customHeight="1">
-      <c r="A41" s="50" t="n"/>
+      <c r="A41" s="49" t="n"/>
       <c r="B41" s="6" t="n"/>
       <c r="C41" s="6" t="n"/>
       <c r="D41" s="6" t="n"/>
@@ -11343,12 +11343,12 @@
       <c r="G41" s="6" t="n"/>
       <c r="H41" s="6" t="n"/>
       <c r="I41" s="6" t="n"/>
-      <c r="J41" s="50" t="n"/>
+      <c r="J41" s="49" t="n"/>
       <c r="K41" s="6" t="n"/>
       <c r="L41" s="6" t="n"/>
     </row>
     <row r="42" ht="18" customHeight="1">
-      <c r="A42" s="50" t="n"/>
+      <c r="A42" s="49" t="n"/>
       <c r="B42" s="6" t="n"/>
       <c r="C42" s="6" t="n"/>
       <c r="D42" s="6" t="n"/>
@@ -11357,12 +11357,12 @@
       <c r="G42" s="6" t="n"/>
       <c r="H42" s="6" t="n"/>
       <c r="I42" s="6" t="n"/>
-      <c r="J42" s="50" t="n"/>
+      <c r="J42" s="49" t="n"/>
       <c r="K42" s="6" t="n"/>
       <c r="L42" s="6" t="n"/>
     </row>
     <row r="43" ht="18" customHeight="1">
-      <c r="A43" s="50" t="n"/>
+      <c r="A43" s="49" t="n"/>
       <c r="B43" s="6" t="n"/>
       <c r="C43" s="6" t="n"/>
       <c r="D43" s="6" t="n"/>
@@ -11371,12 +11371,12 @@
       <c r="G43" s="6" t="n"/>
       <c r="H43" s="6" t="n"/>
       <c r="I43" s="6" t="n"/>
-      <c r="J43" s="50" t="n"/>
+      <c r="J43" s="49" t="n"/>
       <c r="K43" s="6" t="n"/>
       <c r="L43" s="6" t="n"/>
     </row>
     <row r="44" ht="18" customHeight="1">
-      <c r="A44" s="50" t="n"/>
+      <c r="A44" s="49" t="n"/>
       <c r="B44" s="6" t="n"/>
       <c r="C44" s="6" t="n"/>
       <c r="D44" s="6" t="n"/>
@@ -11385,12 +11385,12 @@
       <c r="G44" s="6" t="n"/>
       <c r="H44" s="6" t="n"/>
       <c r="I44" s="6" t="n"/>
-      <c r="J44" s="50" t="n"/>
+      <c r="J44" s="49" t="n"/>
       <c r="K44" s="6" t="n"/>
       <c r="L44" s="6" t="n"/>
     </row>
     <row r="45" ht="18" customHeight="1">
-      <c r="A45" s="50" t="n"/>
+      <c r="A45" s="49" t="n"/>
       <c r="B45" s="6" t="n"/>
       <c r="C45" s="6" t="n"/>
       <c r="D45" s="6" t="n"/>
@@ -11399,12 +11399,12 @@
       <c r="G45" s="6" t="n"/>
       <c r="H45" s="6" t="n"/>
       <c r="I45" s="6" t="n"/>
-      <c r="J45" s="50" t="n"/>
+      <c r="J45" s="49" t="n"/>
       <c r="K45" s="6" t="n"/>
       <c r="L45" s="6" t="n"/>
     </row>
     <row r="46" ht="18" customHeight="1">
-      <c r="A46" s="50" t="n"/>
+      <c r="A46" s="49" t="n"/>
       <c r="B46" s="6" t="n"/>
       <c r="C46" s="6" t="n"/>
       <c r="D46" s="6" t="n"/>
@@ -11413,12 +11413,12 @@
       <c r="G46" s="6" t="n"/>
       <c r="H46" s="6" t="n"/>
       <c r="I46" s="6" t="n"/>
-      <c r="J46" s="50" t="n"/>
+      <c r="J46" s="49" t="n"/>
       <c r="K46" s="6" t="n"/>
       <c r="L46" s="6" t="n"/>
     </row>
     <row r="47" ht="18" customHeight="1">
-      <c r="A47" s="50" t="n"/>
+      <c r="A47" s="49" t="n"/>
       <c r="B47" s="6" t="n"/>
       <c r="C47" s="6" t="n"/>
       <c r="D47" s="6" t="n"/>
@@ -11427,12 +11427,12 @@
       <c r="G47" s="6" t="n"/>
       <c r="H47" s="6" t="n"/>
       <c r="I47" s="6" t="n"/>
-      <c r="J47" s="50" t="n"/>
+      <c r="J47" s="49" t="n"/>
       <c r="K47" s="6" t="n"/>
       <c r="L47" s="6" t="n"/>
     </row>
     <row r="48" ht="18" customHeight="1">
-      <c r="A48" s="50" t="n"/>
+      <c r="A48" s="49" t="n"/>
       <c r="B48" s="6" t="n"/>
       <c r="C48" s="6" t="n"/>
       <c r="D48" s="6" t="n"/>
@@ -11441,12 +11441,12 @@
       <c r="G48" s="6" t="n"/>
       <c r="H48" s="6" t="n"/>
       <c r="I48" s="6" t="n"/>
-      <c r="J48" s="50" t="n"/>
+      <c r="J48" s="49" t="n"/>
       <c r="K48" s="6" t="n"/>
       <c r="L48" s="6" t="n"/>
     </row>
     <row r="49" ht="18" customHeight="1">
-      <c r="A49" s="50" t="n"/>
+      <c r="A49" s="49" t="n"/>
       <c r="B49" s="6" t="n"/>
       <c r="C49" s="6" t="n"/>
       <c r="D49" s="6" t="n"/>
@@ -11455,12 +11455,12 @@
       <c r="G49" s="6" t="n"/>
       <c r="H49" s="6" t="n"/>
       <c r="I49" s="6" t="n"/>
-      <c r="J49" s="50" t="n"/>
+      <c r="J49" s="49" t="n"/>
       <c r="K49" s="6" t="n"/>
       <c r="L49" s="6" t="n"/>
     </row>
     <row r="50" ht="18" customHeight="1">
-      <c r="A50" s="50" t="n"/>
+      <c r="A50" s="49" t="n"/>
       <c r="B50" s="6" t="n"/>
       <c r="C50" s="6" t="n"/>
       <c r="D50" s="6" t="n"/>
@@ -11469,12 +11469,12 @@
       <c r="G50" s="6" t="n"/>
       <c r="H50" s="6" t="n"/>
       <c r="I50" s="6" t="n"/>
-      <c r="J50" s="50" t="n"/>
+      <c r="J50" s="49" t="n"/>
       <c r="K50" s="6" t="n"/>
       <c r="L50" s="6" t="n"/>
     </row>
     <row r="51" ht="18" customHeight="1">
-      <c r="A51" s="50" t="n"/>
+      <c r="A51" s="49" t="n"/>
       <c r="B51" s="6" t="n"/>
       <c r="C51" s="6" t="n"/>
       <c r="D51" s="6" t="n"/>
@@ -11483,12 +11483,12 @@
       <c r="G51" s="6" t="n"/>
       <c r="H51" s="6" t="n"/>
       <c r="I51" s="6" t="n"/>
-      <c r="J51" s="50" t="n"/>
+      <c r="J51" s="49" t="n"/>
       <c r="K51" s="6" t="n"/>
       <c r="L51" s="6" t="n"/>
     </row>
     <row r="52" ht="18" customHeight="1">
-      <c r="A52" s="50" t="n"/>
+      <c r="A52" s="49" t="n"/>
       <c r="B52" s="6" t="n"/>
       <c r="C52" s="6" t="n"/>
       <c r="D52" s="6" t="n"/>
@@ -11497,12 +11497,12 @@
       <c r="G52" s="6" t="n"/>
       <c r="H52" s="6" t="n"/>
       <c r="I52" s="6" t="n"/>
-      <c r="J52" s="50" t="n"/>
+      <c r="J52" s="49" t="n"/>
       <c r="K52" s="6" t="n"/>
       <c r="L52" s="6" t="n"/>
     </row>
     <row r="53" ht="18" customHeight="1">
-      <c r="A53" s="50" t="n"/>
+      <c r="A53" s="49" t="n"/>
       <c r="B53" s="6" t="n"/>
       <c r="C53" s="6" t="n"/>
       <c r="D53" s="6" t="n"/>
@@ -11511,12 +11511,12 @@
       <c r="G53" s="6" t="n"/>
       <c r="H53" s="6" t="n"/>
       <c r="I53" s="6" t="n"/>
-      <c r="J53" s="50" t="n"/>
+      <c r="J53" s="49" t="n"/>
       <c r="K53" s="6" t="n"/>
       <c r="L53" s="6" t="n"/>
     </row>
     <row r="54" ht="18" customHeight="1">
-      <c r="A54" s="50" t="n"/>
+      <c r="A54" s="49" t="n"/>
       <c r="B54" s="6" t="n"/>
       <c r="C54" s="6" t="n"/>
       <c r="D54" s="6" t="n"/>
@@ -11525,12 +11525,12 @@
       <c r="G54" s="6" t="n"/>
       <c r="H54" s="6" t="n"/>
       <c r="I54" s="6" t="n"/>
-      <c r="J54" s="50" t="n"/>
+      <c r="J54" s="49" t="n"/>
       <c r="K54" s="6" t="n"/>
       <c r="L54" s="6" t="n"/>
     </row>
     <row r="55" ht="18" customHeight="1">
-      <c r="A55" s="50" t="n"/>
+      <c r="A55" s="49" t="n"/>
       <c r="B55" s="6" t="n"/>
       <c r="C55" s="6" t="n"/>
       <c r="D55" s="6" t="n"/>
@@ -11539,12 +11539,12 @@
       <c r="G55" s="6" t="n"/>
       <c r="H55" s="6" t="n"/>
       <c r="I55" s="6" t="n"/>
-      <c r="J55" s="50" t="n"/>
+      <c r="J55" s="49" t="n"/>
       <c r="K55" s="6" t="n"/>
       <c r="L55" s="6" t="n"/>
     </row>
     <row r="56" ht="18" customHeight="1">
-      <c r="A56" s="50" t="n"/>
+      <c r="A56" s="49" t="n"/>
       <c r="B56" s="6" t="n"/>
       <c r="C56" s="6" t="n"/>
       <c r="D56" s="6" t="n"/>
@@ -11553,12 +11553,12 @@
       <c r="G56" s="6" t="n"/>
       <c r="H56" s="6" t="n"/>
       <c r="I56" s="6" t="n"/>
-      <c r="J56" s="50" t="n"/>
+      <c r="J56" s="49" t="n"/>
       <c r="K56" s="6" t="n"/>
       <c r="L56" s="6" t="n"/>
     </row>
     <row r="57" ht="18" customHeight="1">
-      <c r="A57" s="50" t="n"/>
+      <c r="A57" s="49" t="n"/>
       <c r="B57" s="6" t="n"/>
       <c r="C57" s="6" t="n"/>
       <c r="D57" s="6" t="n"/>
@@ -11567,12 +11567,12 @@
       <c r="G57" s="6" t="n"/>
       <c r="H57" s="6" t="n"/>
       <c r="I57" s="6" t="n"/>
-      <c r="J57" s="50" t="n"/>
+      <c r="J57" s="49" t="n"/>
       <c r="K57" s="6" t="n"/>
       <c r="L57" s="6" t="n"/>
     </row>
     <row r="58" ht="18" customHeight="1">
-      <c r="A58" s="50" t="n"/>
+      <c r="A58" s="49" t="n"/>
       <c r="B58" s="6" t="n"/>
       <c r="C58" s="6" t="n"/>
       <c r="D58" s="6" t="n"/>
@@ -11581,12 +11581,12 @@
       <c r="G58" s="6" t="n"/>
       <c r="H58" s="6" t="n"/>
       <c r="I58" s="6" t="n"/>
-      <c r="J58" s="50" t="n"/>
+      <c r="J58" s="49" t="n"/>
       <c r="K58" s="6" t="n"/>
       <c r="L58" s="6" t="n"/>
     </row>
     <row r="59" ht="18" customHeight="1">
-      <c r="A59" s="50" t="n"/>
+      <c r="A59" s="49" t="n"/>
       <c r="B59" s="6" t="n"/>
       <c r="C59" s="6" t="n"/>
       <c r="D59" s="6" t="n"/>
@@ -11595,7 +11595,7 @@
       <c r="G59" s="6" t="n"/>
       <c r="H59" s="6" t="n"/>
       <c r="I59" s="6" t="n"/>
-      <c r="J59" s="50" t="n"/>
+      <c r="J59" s="49" t="n"/>
       <c r="K59" s="6" t="n"/>
       <c r="L59" s="6" t="n"/>
     </row>

</xml_diff>